<commit_message>
Restore full content on 10 CNC forms (header, decision, signature)
The engine-graphics rebuild used the minimal log generator, which
dropped the job header, disposition section and signature block — the
forms became a bare table.

Regenerated all 10 with complete sections via the official engine
(form_engine.generate_form + a full-content A4-landscape log builder):
job/reference header, record table, decision/disposition section,
3-column approval signature block, Vietnamese cell-comment guidance on
key fields and columns, and PASS/HOLD/FAIL dropdowns. Content deepened
to a professional inspection-engineering standard. Generator:
_reports/forms/build/gen_v3.py. form_control_registry sha256 refreshed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mom/docs/forms/frm-300-technical/FRM-312_Ballooned_Drawing_Characteristic_Accountability_Sheet.xlsx
+++ b/mom/docs/forms/frm-300-technical/FRM-312_Ballooned_Drawing_Characteristic_Accountability_Sheet.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="83">
+  <fonts count="84">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -474,18 +474,23 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="00334155"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <color rgb="000F172A"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00CBD5E1"/>
       <sz val="8"/>
     </font>
     <font>
@@ -740,14 +745,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00005A9E"/>
-        <bgColor rgb="00005A9E"/>
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00005A9E"/>
+        <bgColor rgb="00005A9E"/>
       </patternFill>
     </fill>
     <fill>
@@ -757,7 +762,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="246">
+  <borders count="257">
     <border>
       <left/>
       <right/>
@@ -3347,6 +3352,7 @@
         <color rgb="000078D4"/>
       </left>
       <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="00E2E8F0"/>
       </bottom>
@@ -3354,6 +3360,7 @@
     <border>
       <left/>
       <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="00E2E8F0"/>
       </bottom>
@@ -3363,6 +3370,7 @@
       <right style="thin">
         <color rgb="00E2E8F0"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="00E2E8F0"/>
       </bottom>
@@ -3372,6 +3380,7 @@
       <right style="thin">
         <color rgb="000078D4"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="00E2E8F0"/>
       </bottom>
@@ -3383,6 +3392,7 @@
       <right style="thin">
         <color rgb="00E2E8F0"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="00E2E8F0"/>
       </bottom>
@@ -3441,6 +3451,7 @@
         <color rgb="000078D4"/>
       </left>
       <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="000078D4"/>
       </bottom>
@@ -3448,6 +3459,7 @@
     <border>
       <left/>
       <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="000078D4"/>
       </bottom>
@@ -3457,6 +3469,7 @@
       <right style="thin">
         <color rgb="00E2E8F0"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="000078D4"/>
       </bottom>
@@ -3466,6 +3479,7 @@
       <right style="thin">
         <color rgb="000078D4"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="000078D4"/>
       </bottom>
@@ -3477,6 +3491,7 @@
       <right style="thin">
         <color rgb="00E2E8F0"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="000078D4"/>
       </bottom>
@@ -3513,14 +3528,120 @@
       <diagonal/>
     </border>
     <border>
-      <right/>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="000078D4"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right/>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="000078D4"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right/>
+      <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="495">
+  <cellXfs count="513">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -4667,51 +4788,97 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="216" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="217" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="79" fillId="49" borderId="222" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="224" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="225" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="220" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="79" fillId="49" borderId="220" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="79" fillId="49" borderId="221" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="221" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="226" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="80" fillId="50" borderId="231" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="231" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="233" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="234" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="81" fillId="47" borderId="229" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="229" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="47" borderId="230" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="229" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="230" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="236" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="81" fillId="51" borderId="229" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="241" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="51" borderId="230" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="80" fillId="50" borderId="241" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="242" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="243" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="81" fillId="51" borderId="239" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="239" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="51" borderId="240" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="239" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="240" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="244" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="82" fillId="48" borderId="213" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="81" fillId="50" borderId="222" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="50" borderId="220" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="50" borderId="221" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="249" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="247" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="47" borderId="245" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="80" fillId="47" borderId="248" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="51" borderId="247" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="51" borderId="248" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="254" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="51" borderId="252" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="51" borderId="253" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="49" borderId="213" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="47" borderId="213" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="214" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="215" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="255" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="235" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="256" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="83" fillId="48" borderId="213" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4788,6 +4955,64 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>QMS</author>
+  </authors>
+  <commentList>
+    <comment ref="A12" authorId="0" shapeId="0">
+      <text>
+        <t>Tổng số đặc tính
+Tổng số bong bóng đã đánh trên bản vẽ.</t>
+      </text>
+    </comment>
+    <comment ref="AC12" authorId="0" shapeId="0">
+      <text>
+        <t>Tham chiếu FAI
+FRM-311 — Báo cáo kiểm tra sản phẩm đầu (First Article).</t>
+      </text>
+    </comment>
+    <comment ref="D15" authorId="0" shapeId="0">
+      <text>
+        <t>Số bong bóng
+Số duy nhất gắn cho mỗi đặc tính trên bản vẽ.</t>
+      </text>
+    </comment>
+    <comment ref="U15" authorId="0" shapeId="0">
+      <text>
+        <t>Quy cách &amp; dung sai
+Giá trị danh nghĩa kèm dung sai hoặc khung GD&amp;T.</t>
+      </text>
+    </comment>
+    <comment ref="AE15" authorId="0" shapeId="0">
+      <text>
+        <t>Phân loại
+CTQ = trọng yếu chất lượng · KPC = đặc tính quá trình then chốt · STD = thường.</t>
+      </text>
+    </comment>
+    <comment ref="AJ15" authorId="0" shapeId="0">
+      <text>
+        <t>Phương pháp kiểm
+Caliper, micrometer, CMM, calíp ren, đo biên dạng…</t>
+      </text>
+    </comment>
+    <comment ref="AY15" authorId="0" shapeId="0">
+      <text>
+        <t>Form ghi nhận
+Form lưu kết quả: FRM-311 (FAI), FRM-622 (in-process)…</t>
+      </text>
+    </comment>
+    <comment ref="A35" authorId="0" shapeId="0">
+      <text>
+        <t>Đã đánh bong bóng đủ?
+Mọi kích thước, ghi chú và GD&amp;T trên bản vẽ phải có một dòng tại đây.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -4811,9 +5036,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5110,7 +5332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:BS27"/>
+  <dimension ref="A2:BD44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.375" customWidth="1" style="264" min="1" max="1"/>
@@ -5425,7 +5647,7 @@
       <c r="BD6" s="30" t="n"/>
     </row>
     <row r="7" ht="4" customHeight="1" s="264">
-      <c r="A7" s="494" t="n"/>
+      <c r="A7" s="469" t="n"/>
       <c r="B7" s="26" t="n"/>
       <c r="C7" s="26" t="n"/>
       <c r="D7" s="26" t="n"/>
@@ -5485,7 +5707,7 @@
     <row r="8" ht="17" customHeight="1" s="264">
       <c r="A8" s="470" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1.  DATA LOG</t>
+          <t xml:space="preserve">  1.  DRAWING &amp; PART HEADER</t>
         </is>
       </c>
       <c r="B8" s="471" t="n"/>
@@ -5544,30 +5766,22 @@
       <c r="BC8" s="471" t="n"/>
       <c r="BD8" s="472" t="n"/>
     </row>
-    <row r="9" ht="17" customHeight="1" s="264">
+    <row r="9" ht="20" customHeight="1" s="264">
       <c r="A9" s="473" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Part No. / Rev</t>
         </is>
       </c>
       <c r="B9" s="474" t="n"/>
       <c r="C9" s="474" t="n"/>
-      <c r="D9" s="475" t="n"/>
-      <c r="E9" s="476" t="inlineStr">
-        <is>
-          <t>Balloon</t>
-        </is>
-      </c>
+      <c r="D9" s="474" t="n"/>
+      <c r="E9" s="474" t="n"/>
       <c r="F9" s="474" t="n"/>
       <c r="G9" s="474" t="n"/>
       <c r="H9" s="474" t="n"/>
-      <c r="I9" s="475" t="n"/>
-      <c r="J9" s="476" t="inlineStr">
-        <is>
-          <t>Feature / Characteristic</t>
-        </is>
-      </c>
-      <c r="K9" s="474" t="n"/>
+      <c r="I9" s="474" t="n"/>
+      <c r="J9" s="475" t="n"/>
+      <c r="K9" s="476" t="n"/>
       <c r="L9" s="474" t="n"/>
       <c r="M9" s="474" t="n"/>
       <c r="N9" s="474" t="n"/>
@@ -5578,36 +5792,28 @@
       <c r="S9" s="474" t="n"/>
       <c r="T9" s="474" t="n"/>
       <c r="U9" s="474" t="n"/>
-      <c r="V9" s="475" t="n"/>
-      <c r="W9" s="476" t="inlineStr">
-        <is>
-          <t>Spec / Tolerance</t>
-        </is>
-      </c>
+      <c r="V9" s="474" t="n"/>
+      <c r="W9" s="474" t="n"/>
       <c r="X9" s="474" t="n"/>
       <c r="Y9" s="474" t="n"/>
       <c r="Z9" s="474" t="n"/>
       <c r="AA9" s="474" t="n"/>
-      <c r="AB9" s="474" t="n"/>
-      <c r="AC9" s="474" t="n"/>
+      <c r="AB9" s="475" t="n"/>
+      <c r="AC9" s="477" t="inlineStr">
+        <is>
+          <t>Drawing No. / Rev</t>
+        </is>
+      </c>
       <c r="AD9" s="474" t="n"/>
       <c r="AE9" s="474" t="n"/>
       <c r="AF9" s="474" t="n"/>
-      <c r="AG9" s="475" t="n"/>
-      <c r="AH9" s="476" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
+      <c r="AG9" s="474" t="n"/>
+      <c r="AH9" s="474" t="n"/>
       <c r="AI9" s="474" t="n"/>
       <c r="AJ9" s="474" t="n"/>
       <c r="AK9" s="474" t="n"/>
       <c r="AL9" s="475" t="n"/>
-      <c r="AM9" s="476" t="inlineStr">
-        <is>
-          <t>Inspection Method</t>
-        </is>
-      </c>
+      <c r="AM9" s="478" t="n"/>
       <c r="AN9" s="474" t="n"/>
       <c r="AO9" s="474" t="n"/>
       <c r="AP9" s="474" t="n"/>
@@ -5615,1265 +5821,2350 @@
       <c r="AR9" s="474" t="n"/>
       <c r="AS9" s="474" t="n"/>
       <c r="AT9" s="474" t="n"/>
-      <c r="AU9" s="475" t="n"/>
-      <c r="AV9" s="476" t="inlineStr">
-        <is>
-          <t>Sample Plan</t>
-        </is>
-      </c>
+      <c r="AU9" s="474" t="n"/>
+      <c r="AV9" s="474" t="n"/>
       <c r="AW9" s="474" t="n"/>
       <c r="AX9" s="474" t="n"/>
       <c r="AY9" s="474" t="n"/>
-      <c r="AZ9" s="475" t="n"/>
-      <c r="BA9" s="477" t="inlineStr">
-        <is>
-          <t>Form Ref</t>
-        </is>
-      </c>
+      <c r="AZ9" s="474" t="n"/>
+      <c r="BA9" s="474" t="n"/>
       <c r="BB9" s="474" t="n"/>
       <c r="BC9" s="474" t="n"/>
-      <c r="BD9" s="478" t="n"/>
+      <c r="BD9" s="479" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1" s="264">
-      <c r="A10" s="479" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="480" t="n"/>
-      <c r="C10" s="480" t="n"/>
+      <c r="A10" s="480" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B10" s="481" t="n"/>
+      <c r="C10" s="481" t="n"/>
       <c r="D10" s="481" t="n"/>
-      <c r="E10" s="482" t="n"/>
-      <c r="F10" s="480" t="n"/>
-      <c r="G10" s="480" t="n"/>
-      <c r="H10" s="480" t="n"/>
+      <c r="E10" s="481" t="n"/>
+      <c r="F10" s="481" t="n"/>
+      <c r="G10" s="481" t="n"/>
+      <c r="H10" s="481" t="n"/>
       <c r="I10" s="481" t="n"/>
       <c r="J10" s="482" t="n"/>
-      <c r="K10" s="480" t="n"/>
-      <c r="L10" s="480" t="n"/>
-      <c r="M10" s="480" t="n"/>
-      <c r="N10" s="480" t="n"/>
-      <c r="O10" s="480" t="n"/>
-      <c r="P10" s="480" t="n"/>
-      <c r="Q10" s="480" t="n"/>
-      <c r="R10" s="480" t="n"/>
-      <c r="S10" s="480" t="n"/>
-      <c r="T10" s="480" t="n"/>
-      <c r="U10" s="480" t="n"/>
+      <c r="K10" s="483" t="n"/>
+      <c r="L10" s="481" t="n"/>
+      <c r="M10" s="481" t="n"/>
+      <c r="N10" s="481" t="n"/>
+      <c r="O10" s="481" t="n"/>
+      <c r="P10" s="481" t="n"/>
+      <c r="Q10" s="481" t="n"/>
+      <c r="R10" s="481" t="n"/>
+      <c r="S10" s="481" t="n"/>
+      <c r="T10" s="481" t="n"/>
+      <c r="U10" s="481" t="n"/>
       <c r="V10" s="481" t="n"/>
-      <c r="W10" s="482" t="n"/>
-      <c r="X10" s="480" t="n"/>
-      <c r="Y10" s="480" t="n"/>
-      <c r="Z10" s="480" t="n"/>
-      <c r="AA10" s="480" t="n"/>
-      <c r="AB10" s="480" t="n"/>
-      <c r="AC10" s="480" t="n"/>
-      <c r="AD10" s="480" t="n"/>
-      <c r="AE10" s="480" t="n"/>
-      <c r="AF10" s="480" t="n"/>
+      <c r="W10" s="481" t="n"/>
+      <c r="X10" s="481" t="n"/>
+      <c r="Y10" s="481" t="n"/>
+      <c r="Z10" s="481" t="n"/>
+      <c r="AA10" s="481" t="n"/>
+      <c r="AB10" s="482" t="n"/>
+      <c r="AC10" s="484" t="inlineStr">
+        <is>
+          <t>Job / WO</t>
+        </is>
+      </c>
+      <c r="AD10" s="481" t="n"/>
+      <c r="AE10" s="481" t="n"/>
+      <c r="AF10" s="481" t="n"/>
       <c r="AG10" s="481" t="n"/>
-      <c r="AH10" s="482" t="n"/>
-      <c r="AI10" s="480" t="n"/>
-      <c r="AJ10" s="480" t="n"/>
-      <c r="AK10" s="480" t="n"/>
-      <c r="AL10" s="481" t="n"/>
-      <c r="AM10" s="482" t="n"/>
-      <c r="AN10" s="480" t="n"/>
-      <c r="AO10" s="480" t="n"/>
-      <c r="AP10" s="480" t="n"/>
-      <c r="AQ10" s="480" t="n"/>
-      <c r="AR10" s="480" t="n"/>
-      <c r="AS10" s="480" t="n"/>
-      <c r="AT10" s="480" t="n"/>
+      <c r="AH10" s="481" t="n"/>
+      <c r="AI10" s="481" t="n"/>
+      <c r="AJ10" s="481" t="n"/>
+      <c r="AK10" s="481" t="n"/>
+      <c r="AL10" s="482" t="n"/>
+      <c r="AM10" s="485" t="n"/>
+      <c r="AN10" s="481" t="n"/>
+      <c r="AO10" s="481" t="n"/>
+      <c r="AP10" s="481" t="n"/>
+      <c r="AQ10" s="481" t="n"/>
+      <c r="AR10" s="481" t="n"/>
+      <c r="AS10" s="481" t="n"/>
+      <c r="AT10" s="481" t="n"/>
       <c r="AU10" s="481" t="n"/>
-      <c r="AV10" s="482" t="n"/>
-      <c r="AW10" s="480" t="n"/>
-      <c r="AX10" s="480" t="n"/>
-      <c r="AY10" s="480" t="n"/>
+      <c r="AV10" s="481" t="n"/>
+      <c r="AW10" s="481" t="n"/>
+      <c r="AX10" s="481" t="n"/>
+      <c r="AY10" s="481" t="n"/>
       <c r="AZ10" s="481" t="n"/>
-      <c r="BA10" s="483" t="n"/>
-      <c r="BB10" s="480" t="n"/>
-      <c r="BC10" s="480" t="n"/>
-      <c r="BD10" s="484" t="n"/>
+      <c r="BA10" s="481" t="n"/>
+      <c r="BB10" s="481" t="n"/>
+      <c r="BC10" s="481" t="n"/>
+      <c r="BD10" s="486" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1" s="264">
-      <c r="A11" s="479" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="480" t="n"/>
-      <c r="C11" s="480" t="n"/>
+      <c r="A11" s="480" t="inlineStr">
+        <is>
+          <t>Prepared By</t>
+        </is>
+      </c>
+      <c r="B11" s="481" t="n"/>
+      <c r="C11" s="481" t="n"/>
       <c r="D11" s="481" t="n"/>
-      <c r="E11" s="485" t="n"/>
-      <c r="F11" s="480" t="n"/>
-      <c r="G11" s="480" t="n"/>
-      <c r="H11" s="480" t="n"/>
+      <c r="E11" s="481" t="n"/>
+      <c r="F11" s="481" t="n"/>
+      <c r="G11" s="481" t="n"/>
+      <c r="H11" s="481" t="n"/>
       <c r="I11" s="481" t="n"/>
-      <c r="J11" s="485" t="n"/>
-      <c r="K11" s="480" t="n"/>
-      <c r="L11" s="480" t="n"/>
-      <c r="M11" s="480" t="n"/>
-      <c r="N11" s="480" t="n"/>
-      <c r="O11" s="480" t="n"/>
-      <c r="P11" s="480" t="n"/>
-      <c r="Q11" s="480" t="n"/>
-      <c r="R11" s="480" t="n"/>
-      <c r="S11" s="480" t="n"/>
-      <c r="T11" s="480" t="n"/>
-      <c r="U11" s="480" t="n"/>
+      <c r="J11" s="482" t="n"/>
+      <c r="K11" s="483" t="n"/>
+      <c r="L11" s="481" t="n"/>
+      <c r="M11" s="481" t="n"/>
+      <c r="N11" s="481" t="n"/>
+      <c r="O11" s="481" t="n"/>
+      <c r="P11" s="481" t="n"/>
+      <c r="Q11" s="481" t="n"/>
+      <c r="R11" s="481" t="n"/>
+      <c r="S11" s="481" t="n"/>
+      <c r="T11" s="481" t="n"/>
+      <c r="U11" s="481" t="n"/>
       <c r="V11" s="481" t="n"/>
-      <c r="W11" s="485" t="n"/>
-      <c r="X11" s="480" t="n"/>
-      <c r="Y11" s="480" t="n"/>
-      <c r="Z11" s="480" t="n"/>
-      <c r="AA11" s="480" t="n"/>
-      <c r="AB11" s="480" t="n"/>
-      <c r="AC11" s="480" t="n"/>
-      <c r="AD11" s="480" t="n"/>
-      <c r="AE11" s="480" t="n"/>
-      <c r="AF11" s="480" t="n"/>
+      <c r="W11" s="481" t="n"/>
+      <c r="X11" s="481" t="n"/>
+      <c r="Y11" s="481" t="n"/>
+      <c r="Z11" s="481" t="n"/>
+      <c r="AA11" s="481" t="n"/>
+      <c r="AB11" s="482" t="n"/>
+      <c r="AC11" s="484" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="AD11" s="481" t="n"/>
+      <c r="AE11" s="481" t="n"/>
+      <c r="AF11" s="481" t="n"/>
       <c r="AG11" s="481" t="n"/>
-      <c r="AH11" s="485" t="n"/>
-      <c r="AI11" s="480" t="n"/>
-      <c r="AJ11" s="480" t="n"/>
-      <c r="AK11" s="480" t="n"/>
-      <c r="AL11" s="481" t="n"/>
+      <c r="AH11" s="481" t="n"/>
+      <c r="AI11" s="481" t="n"/>
+      <c r="AJ11" s="481" t="n"/>
+      <c r="AK11" s="481" t="n"/>
+      <c r="AL11" s="482" t="n"/>
       <c r="AM11" s="485" t="n"/>
-      <c r="AN11" s="480" t="n"/>
-      <c r="AO11" s="480" t="n"/>
-      <c r="AP11" s="480" t="n"/>
-      <c r="AQ11" s="480" t="n"/>
-      <c r="AR11" s="480" t="n"/>
-      <c r="AS11" s="480" t="n"/>
-      <c r="AT11" s="480" t="n"/>
+      <c r="AN11" s="481" t="n"/>
+      <c r="AO11" s="481" t="n"/>
+      <c r="AP11" s="481" t="n"/>
+      <c r="AQ11" s="481" t="n"/>
+      <c r="AR11" s="481" t="n"/>
+      <c r="AS11" s="481" t="n"/>
+      <c r="AT11" s="481" t="n"/>
       <c r="AU11" s="481" t="n"/>
-      <c r="AV11" s="485" t="n"/>
-      <c r="AW11" s="480" t="n"/>
-      <c r="AX11" s="480" t="n"/>
-      <c r="AY11" s="480" t="n"/>
+      <c r="AV11" s="481" t="n"/>
+      <c r="AW11" s="481" t="n"/>
+      <c r="AX11" s="481" t="n"/>
+      <c r="AY11" s="481" t="n"/>
       <c r="AZ11" s="481" t="n"/>
-      <c r="BA11" s="486" t="n"/>
-      <c r="BB11" s="480" t="n"/>
-      <c r="BC11" s="480" t="n"/>
-      <c r="BD11" s="484" t="n"/>
+      <c r="BA11" s="481" t="n"/>
+      <c r="BB11" s="481" t="n"/>
+      <c r="BC11" s="481" t="n"/>
+      <c r="BD11" s="486" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1" s="264">
-      <c r="A12" s="479" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="480" t="n"/>
-      <c r="C12" s="480" t="n"/>
-      <c r="D12" s="481" t="n"/>
-      <c r="E12" s="482" t="n"/>
-      <c r="F12" s="480" t="n"/>
-      <c r="G12" s="480" t="n"/>
-      <c r="H12" s="480" t="n"/>
-      <c r="I12" s="481" t="n"/>
-      <c r="J12" s="482" t="n"/>
-      <c r="K12" s="480" t="n"/>
-      <c r="L12" s="480" t="n"/>
-      <c r="M12" s="480" t="n"/>
-      <c r="N12" s="480" t="n"/>
-      <c r="O12" s="480" t="n"/>
-      <c r="P12" s="480" t="n"/>
-      <c r="Q12" s="480" t="n"/>
-      <c r="R12" s="480" t="n"/>
-      <c r="S12" s="480" t="n"/>
-      <c r="T12" s="480" t="n"/>
-      <c r="U12" s="480" t="n"/>
-      <c r="V12" s="481" t="n"/>
-      <c r="W12" s="482" t="n"/>
-      <c r="X12" s="480" t="n"/>
-      <c r="Y12" s="480" t="n"/>
-      <c r="Z12" s="480" t="n"/>
-      <c r="AA12" s="480" t="n"/>
-      <c r="AB12" s="480" t="n"/>
-      <c r="AC12" s="480" t="n"/>
-      <c r="AD12" s="480" t="n"/>
-      <c r="AE12" s="480" t="n"/>
-      <c r="AF12" s="480" t="n"/>
-      <c r="AG12" s="481" t="n"/>
-      <c r="AH12" s="482" t="n"/>
-      <c r="AI12" s="480" t="n"/>
-      <c r="AJ12" s="480" t="n"/>
-      <c r="AK12" s="480" t="n"/>
-      <c r="AL12" s="481" t="n"/>
-      <c r="AM12" s="482" t="n"/>
-      <c r="AN12" s="480" t="n"/>
-      <c r="AO12" s="480" t="n"/>
-      <c r="AP12" s="480" t="n"/>
-      <c r="AQ12" s="480" t="n"/>
-      <c r="AR12" s="480" t="n"/>
-      <c r="AS12" s="480" t="n"/>
-      <c r="AT12" s="480" t="n"/>
-      <c r="AU12" s="481" t="n"/>
-      <c r="AV12" s="482" t="n"/>
-      <c r="AW12" s="480" t="n"/>
-      <c r="AX12" s="480" t="n"/>
-      <c r="AY12" s="480" t="n"/>
-      <c r="AZ12" s="481" t="n"/>
-      <c r="BA12" s="483" t="n"/>
-      <c r="BB12" s="480" t="n"/>
-      <c r="BC12" s="480" t="n"/>
-      <c r="BD12" s="484" t="n"/>
+      <c r="A12" s="487" t="inlineStr">
+        <is>
+          <t>Total Characteristics</t>
+        </is>
+      </c>
+      <c r="B12" s="488" t="n"/>
+      <c r="C12" s="488" t="n"/>
+      <c r="D12" s="488" t="n"/>
+      <c r="E12" s="488" t="n"/>
+      <c r="F12" s="488" t="n"/>
+      <c r="G12" s="488" t="n"/>
+      <c r="H12" s="488" t="n"/>
+      <c r="I12" s="488" t="n"/>
+      <c r="J12" s="489" t="n"/>
+      <c r="K12" s="490" t="n"/>
+      <c r="L12" s="488" t="n"/>
+      <c r="M12" s="488" t="n"/>
+      <c r="N12" s="488" t="n"/>
+      <c r="O12" s="488" t="n"/>
+      <c r="P12" s="488" t="n"/>
+      <c r="Q12" s="488" t="n"/>
+      <c r="R12" s="488" t="n"/>
+      <c r="S12" s="488" t="n"/>
+      <c r="T12" s="488" t="n"/>
+      <c r="U12" s="488" t="n"/>
+      <c r="V12" s="488" t="n"/>
+      <c r="W12" s="488" t="n"/>
+      <c r="X12" s="488" t="n"/>
+      <c r="Y12" s="488" t="n"/>
+      <c r="Z12" s="488" t="n"/>
+      <c r="AA12" s="488" t="n"/>
+      <c r="AB12" s="489" t="n"/>
+      <c r="AC12" s="491" t="inlineStr">
+        <is>
+          <t>Linked FRM-311 FAI</t>
+        </is>
+      </c>
+      <c r="AD12" s="488" t="n"/>
+      <c r="AE12" s="488" t="n"/>
+      <c r="AF12" s="488" t="n"/>
+      <c r="AG12" s="488" t="n"/>
+      <c r="AH12" s="488" t="n"/>
+      <c r="AI12" s="488" t="n"/>
+      <c r="AJ12" s="488" t="n"/>
+      <c r="AK12" s="488" t="n"/>
+      <c r="AL12" s="489" t="n"/>
+      <c r="AM12" s="492" t="n"/>
+      <c r="AN12" s="488" t="n"/>
+      <c r="AO12" s="488" t="n"/>
+      <c r="AP12" s="488" t="n"/>
+      <c r="AQ12" s="488" t="n"/>
+      <c r="AR12" s="488" t="n"/>
+      <c r="AS12" s="488" t="n"/>
+      <c r="AT12" s="488" t="n"/>
+      <c r="AU12" s="488" t="n"/>
+      <c r="AV12" s="488" t="n"/>
+      <c r="AW12" s="488" t="n"/>
+      <c r="AX12" s="488" t="n"/>
+      <c r="AY12" s="488" t="n"/>
+      <c r="AZ12" s="488" t="n"/>
+      <c r="BA12" s="488" t="n"/>
+      <c r="BB12" s="488" t="n"/>
+      <c r="BC12" s="488" t="n"/>
+      <c r="BD12" s="493" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1" s="264">
-      <c r="A13" s="479" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="480" t="n"/>
-      <c r="C13" s="480" t="n"/>
-      <c r="D13" s="481" t="n"/>
-      <c r="E13" s="485" t="n"/>
-      <c r="F13" s="480" t="n"/>
-      <c r="G13" s="480" t="n"/>
-      <c r="H13" s="480" t="n"/>
-      <c r="I13" s="481" t="n"/>
-      <c r="J13" s="485" t="n"/>
-      <c r="K13" s="480" t="n"/>
-      <c r="L13" s="480" t="n"/>
-      <c r="M13" s="480" t="n"/>
-      <c r="N13" s="480" t="n"/>
-      <c r="O13" s="480" t="n"/>
-      <c r="P13" s="480" t="n"/>
-      <c r="Q13" s="480" t="n"/>
-      <c r="R13" s="480" t="n"/>
-      <c r="S13" s="480" t="n"/>
-      <c r="T13" s="480" t="n"/>
-      <c r="U13" s="480" t="n"/>
-      <c r="V13" s="481" t="n"/>
-      <c r="W13" s="485" t="n"/>
-      <c r="X13" s="480" t="n"/>
-      <c r="Y13" s="480" t="n"/>
-      <c r="Z13" s="480" t="n"/>
-      <c r="AA13" s="480" t="n"/>
-      <c r="AB13" s="480" t="n"/>
-      <c r="AC13" s="480" t="n"/>
-      <c r="AD13" s="480" t="n"/>
-      <c r="AE13" s="480" t="n"/>
-      <c r="AF13" s="480" t="n"/>
-      <c r="AG13" s="481" t="n"/>
-      <c r="AH13" s="485" t="n"/>
-      <c r="AI13" s="480" t="n"/>
-      <c r="AJ13" s="480" t="n"/>
-      <c r="AK13" s="480" t="n"/>
-      <c r="AL13" s="481" t="n"/>
-      <c r="AM13" s="485" t="n"/>
-      <c r="AN13" s="480" t="n"/>
-      <c r="AO13" s="480" t="n"/>
-      <c r="AP13" s="480" t="n"/>
-      <c r="AQ13" s="480" t="n"/>
-      <c r="AR13" s="480" t="n"/>
-      <c r="AS13" s="480" t="n"/>
-      <c r="AT13" s="480" t="n"/>
-      <c r="AU13" s="481" t="n"/>
-      <c r="AV13" s="485" t="n"/>
-      <c r="AW13" s="480" t="n"/>
-      <c r="AX13" s="480" t="n"/>
-      <c r="AY13" s="480" t="n"/>
-      <c r="AZ13" s="481" t="n"/>
-      <c r="BA13" s="486" t="n"/>
-      <c r="BB13" s="480" t="n"/>
-      <c r="BC13" s="480" t="n"/>
-      <c r="BD13" s="484" t="n"/>
+    <row r="13" ht="4" customHeight="1" s="264">
+      <c r="A13" s="469" t="n"/>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26" t="n"/>
+      <c r="H13" s="26" t="n"/>
+      <c r="I13" s="26" t="n"/>
+      <c r="J13" s="26" t="n"/>
+      <c r="K13" s="26" t="n"/>
+      <c r="L13" s="26" t="n"/>
+      <c r="M13" s="26" t="n"/>
+      <c r="N13" s="26" t="n"/>
+      <c r="O13" s="26" t="n"/>
+      <c r="P13" s="26" t="n"/>
+      <c r="Q13" s="26" t="n"/>
+      <c r="R13" s="26" t="n"/>
+      <c r="S13" s="26" t="n"/>
+      <c r="T13" s="26" t="n"/>
+      <c r="U13" s="26" t="n"/>
+      <c r="V13" s="26" t="n"/>
+      <c r="W13" s="26" t="n"/>
+      <c r="X13" s="26" t="n"/>
+      <c r="Y13" s="26" t="n"/>
+      <c r="Z13" s="26" t="n"/>
+      <c r="AA13" s="26" t="n"/>
+      <c r="AB13" s="26" t="n"/>
+      <c r="AC13" s="26" t="n"/>
+      <c r="AD13" s="26" t="n"/>
+      <c r="AE13" s="26" t="n"/>
+      <c r="AF13" s="26" t="n"/>
+      <c r="AG13" s="26" t="n"/>
+      <c r="AH13" s="26" t="n"/>
+      <c r="AI13" s="26" t="n"/>
+      <c r="AJ13" s="26" t="n"/>
+      <c r="AK13" s="26" t="n"/>
+      <c r="AL13" s="26" t="n"/>
+      <c r="AM13" s="26" t="n"/>
+      <c r="AN13" s="26" t="n"/>
+      <c r="AO13" s="26" t="n"/>
+      <c r="AP13" s="26" t="n"/>
+      <c r="AQ13" s="26" t="n"/>
+      <c r="AR13" s="26" t="n"/>
+      <c r="AS13" s="26" t="n"/>
+      <c r="AT13" s="26" t="n"/>
+      <c r="AU13" s="26" t="n"/>
+      <c r="AV13" s="26" t="n"/>
+      <c r="AW13" s="26" t="n"/>
+      <c r="AX13" s="26" t="n"/>
+      <c r="AY13" s="26" t="n"/>
+      <c r="AZ13" s="26" t="n"/>
+      <c r="BA13" s="26" t="n"/>
+      <c r="BB13" s="26" t="n"/>
+      <c r="BC13" s="26" t="n"/>
+      <c r="BD13" s="26" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1" s="264">
-      <c r="A14" s="479" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="480" t="n"/>
-      <c r="C14" s="480" t="n"/>
-      <c r="D14" s="481" t="n"/>
-      <c r="E14" s="482" t="n"/>
-      <c r="F14" s="480" t="n"/>
-      <c r="G14" s="480" t="n"/>
-      <c r="H14" s="480" t="n"/>
-      <c r="I14" s="481" t="n"/>
-      <c r="J14" s="482" t="n"/>
-      <c r="K14" s="480" t="n"/>
-      <c r="L14" s="480" t="n"/>
-      <c r="M14" s="480" t="n"/>
-      <c r="N14" s="480" t="n"/>
-      <c r="O14" s="480" t="n"/>
-      <c r="P14" s="480" t="n"/>
-      <c r="Q14" s="480" t="n"/>
-      <c r="R14" s="480" t="n"/>
-      <c r="S14" s="480" t="n"/>
-      <c r="T14" s="480" t="n"/>
-      <c r="U14" s="480" t="n"/>
-      <c r="V14" s="481" t="n"/>
-      <c r="W14" s="482" t="n"/>
-      <c r="X14" s="480" t="n"/>
-      <c r="Y14" s="480" t="n"/>
-      <c r="Z14" s="480" t="n"/>
-      <c r="AA14" s="480" t="n"/>
-      <c r="AB14" s="480" t="n"/>
-      <c r="AC14" s="480" t="n"/>
-      <c r="AD14" s="480" t="n"/>
-      <c r="AE14" s="480" t="n"/>
-      <c r="AF14" s="480" t="n"/>
-      <c r="AG14" s="481" t="n"/>
-      <c r="AH14" s="482" t="n"/>
-      <c r="AI14" s="480" t="n"/>
-      <c r="AJ14" s="480" t="n"/>
-      <c r="AK14" s="480" t="n"/>
-      <c r="AL14" s="481" t="n"/>
-      <c r="AM14" s="482" t="n"/>
-      <c r="AN14" s="480" t="n"/>
-      <c r="AO14" s="480" t="n"/>
-      <c r="AP14" s="480" t="n"/>
-      <c r="AQ14" s="480" t="n"/>
-      <c r="AR14" s="480" t="n"/>
-      <c r="AS14" s="480" t="n"/>
-      <c r="AT14" s="480" t="n"/>
-      <c r="AU14" s="481" t="n"/>
-      <c r="AV14" s="482" t="n"/>
-      <c r="AW14" s="480" t="n"/>
-      <c r="AX14" s="480" t="n"/>
-      <c r="AY14" s="480" t="n"/>
-      <c r="AZ14" s="481" t="n"/>
-      <c r="BA14" s="483" t="n"/>
-      <c r="BB14" s="480" t="n"/>
-      <c r="BC14" s="480" t="n"/>
-      <c r="BD14" s="484" t="n"/>
+    <row r="14" ht="17" customHeight="1" s="264">
+      <c r="A14" s="470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.  CHARACTERISTIC ACCOUNTABILITY REGISTER</t>
+        </is>
+      </c>
+      <c r="B14" s="471" t="n"/>
+      <c r="C14" s="471" t="n"/>
+      <c r="D14" s="471" t="n"/>
+      <c r="E14" s="471" t="n"/>
+      <c r="F14" s="471" t="n"/>
+      <c r="G14" s="471" t="n"/>
+      <c r="H14" s="471" t="n"/>
+      <c r="I14" s="471" t="n"/>
+      <c r="J14" s="471" t="n"/>
+      <c r="K14" s="471" t="n"/>
+      <c r="L14" s="471" t="n"/>
+      <c r="M14" s="471" t="n"/>
+      <c r="N14" s="471" t="n"/>
+      <c r="O14" s="471" t="n"/>
+      <c r="P14" s="471" t="n"/>
+      <c r="Q14" s="471" t="n"/>
+      <c r="R14" s="471" t="n"/>
+      <c r="S14" s="471" t="n"/>
+      <c r="T14" s="471" t="n"/>
+      <c r="U14" s="471" t="n"/>
+      <c r="V14" s="471" t="n"/>
+      <c r="W14" s="471" t="n"/>
+      <c r="X14" s="471" t="n"/>
+      <c r="Y14" s="471" t="n"/>
+      <c r="Z14" s="471" t="n"/>
+      <c r="AA14" s="471" t="n"/>
+      <c r="AB14" s="471" t="n"/>
+      <c r="AC14" s="471" t="n"/>
+      <c r="AD14" s="471" t="n"/>
+      <c r="AE14" s="471" t="n"/>
+      <c r="AF14" s="471" t="n"/>
+      <c r="AG14" s="471" t="n"/>
+      <c r="AH14" s="471" t="n"/>
+      <c r="AI14" s="471" t="n"/>
+      <c r="AJ14" s="471" t="n"/>
+      <c r="AK14" s="471" t="n"/>
+      <c r="AL14" s="471" t="n"/>
+      <c r="AM14" s="471" t="n"/>
+      <c r="AN14" s="471" t="n"/>
+      <c r="AO14" s="471" t="n"/>
+      <c r="AP14" s="471" t="n"/>
+      <c r="AQ14" s="471" t="n"/>
+      <c r="AR14" s="471" t="n"/>
+      <c r="AS14" s="471" t="n"/>
+      <c r="AT14" s="471" t="n"/>
+      <c r="AU14" s="471" t="n"/>
+      <c r="AV14" s="471" t="n"/>
+      <c r="AW14" s="471" t="n"/>
+      <c r="AX14" s="471" t="n"/>
+      <c r="AY14" s="471" t="n"/>
+      <c r="AZ14" s="471" t="n"/>
+      <c r="BA14" s="471" t="n"/>
+      <c r="BB14" s="471" t="n"/>
+      <c r="BC14" s="471" t="n"/>
+      <c r="BD14" s="472" t="n"/>
     </row>
-    <row r="15" ht="20" customHeight="1" s="264">
-      <c r="A15" s="479" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="480" t="n"/>
-      <c r="C15" s="480" t="n"/>
-      <c r="D15" s="481" t="n"/>
-      <c r="E15" s="485" t="n"/>
-      <c r="F15" s="480" t="n"/>
-      <c r="G15" s="480" t="n"/>
-      <c r="H15" s="480" t="n"/>
-      <c r="I15" s="481" t="n"/>
-      <c r="J15" s="485" t="n"/>
-      <c r="K15" s="480" t="n"/>
-      <c r="L15" s="480" t="n"/>
-      <c r="M15" s="480" t="n"/>
-      <c r="N15" s="480" t="n"/>
-      <c r="O15" s="480" t="n"/>
-      <c r="P15" s="480" t="n"/>
-      <c r="Q15" s="480" t="n"/>
-      <c r="R15" s="480" t="n"/>
-      <c r="S15" s="480" t="n"/>
-      <c r="T15" s="480" t="n"/>
-      <c r="U15" s="480" t="n"/>
-      <c r="V15" s="481" t="n"/>
-      <c r="W15" s="485" t="n"/>
-      <c r="X15" s="480" t="n"/>
-      <c r="Y15" s="480" t="n"/>
-      <c r="Z15" s="480" t="n"/>
-      <c r="AA15" s="480" t="n"/>
-      <c r="AB15" s="480" t="n"/>
-      <c r="AC15" s="480" t="n"/>
-      <c r="AD15" s="480" t="n"/>
-      <c r="AE15" s="480" t="n"/>
-      <c r="AF15" s="480" t="n"/>
-      <c r="AG15" s="481" t="n"/>
-      <c r="AH15" s="485" t="n"/>
-      <c r="AI15" s="480" t="n"/>
-      <c r="AJ15" s="480" t="n"/>
-      <c r="AK15" s="480" t="n"/>
-      <c r="AL15" s="481" t="n"/>
-      <c r="AM15" s="485" t="n"/>
-      <c r="AN15" s="480" t="n"/>
-      <c r="AO15" s="480" t="n"/>
-      <c r="AP15" s="480" t="n"/>
-      <c r="AQ15" s="480" t="n"/>
-      <c r="AR15" s="480" t="n"/>
-      <c r="AS15" s="480" t="n"/>
-      <c r="AT15" s="480" t="n"/>
-      <c r="AU15" s="481" t="n"/>
-      <c r="AV15" s="485" t="n"/>
-      <c r="AW15" s="480" t="n"/>
-      <c r="AX15" s="480" t="n"/>
-      <c r="AY15" s="480" t="n"/>
-      <c r="AZ15" s="481" t="n"/>
-      <c r="BA15" s="486" t="n"/>
-      <c r="BB15" s="480" t="n"/>
-      <c r="BC15" s="480" t="n"/>
-      <c r="BD15" s="484" t="n"/>
+    <row r="15" ht="17" customHeight="1" s="264">
+      <c r="A15" s="494" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B15" s="474" t="n"/>
+      <c r="C15" s="475" t="n"/>
+      <c r="D15" s="495" t="inlineStr">
+        <is>
+          <t>Balloon</t>
+        </is>
+      </c>
+      <c r="E15" s="474" t="n"/>
+      <c r="F15" s="474" t="n"/>
+      <c r="G15" s="475" t="n"/>
+      <c r="H15" s="495" t="inlineStr">
+        <is>
+          <t>Feature / Characteristic</t>
+        </is>
+      </c>
+      <c r="I15" s="474" t="n"/>
+      <c r="J15" s="474" t="n"/>
+      <c r="K15" s="474" t="n"/>
+      <c r="L15" s="474" t="n"/>
+      <c r="M15" s="474" t="n"/>
+      <c r="N15" s="474" t="n"/>
+      <c r="O15" s="474" t="n"/>
+      <c r="P15" s="474" t="n"/>
+      <c r="Q15" s="474" t="n"/>
+      <c r="R15" s="474" t="n"/>
+      <c r="S15" s="474" t="n"/>
+      <c r="T15" s="475" t="n"/>
+      <c r="U15" s="495" t="inlineStr">
+        <is>
+          <t>Spec &amp; Tolerance</t>
+        </is>
+      </c>
+      <c r="V15" s="474" t="n"/>
+      <c r="W15" s="474" t="n"/>
+      <c r="X15" s="474" t="n"/>
+      <c r="Y15" s="474" t="n"/>
+      <c r="Z15" s="474" t="n"/>
+      <c r="AA15" s="474" t="n"/>
+      <c r="AB15" s="474" t="n"/>
+      <c r="AC15" s="474" t="n"/>
+      <c r="AD15" s="475" t="n"/>
+      <c r="AE15" s="495" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="AF15" s="474" t="n"/>
+      <c r="AG15" s="474" t="n"/>
+      <c r="AH15" s="474" t="n"/>
+      <c r="AI15" s="475" t="n"/>
+      <c r="AJ15" s="495" t="inlineStr">
+        <is>
+          <t>Inspection Method</t>
+        </is>
+      </c>
+      <c r="AK15" s="474" t="n"/>
+      <c r="AL15" s="474" t="n"/>
+      <c r="AM15" s="474" t="n"/>
+      <c r="AN15" s="474" t="n"/>
+      <c r="AO15" s="474" t="n"/>
+      <c r="AP15" s="474" t="n"/>
+      <c r="AQ15" s="474" t="n"/>
+      <c r="AR15" s="475" t="n"/>
+      <c r="AS15" s="495" t="inlineStr">
+        <is>
+          <t>Gage / Equipment</t>
+        </is>
+      </c>
+      <c r="AT15" s="474" t="n"/>
+      <c r="AU15" s="474" t="n"/>
+      <c r="AV15" s="474" t="n"/>
+      <c r="AW15" s="474" t="n"/>
+      <c r="AX15" s="475" t="n"/>
+      <c r="AY15" s="496" t="inlineStr">
+        <is>
+          <t>Record Form</t>
+        </is>
+      </c>
+      <c r="AZ15" s="474" t="n"/>
+      <c r="BA15" s="474" t="n"/>
+      <c r="BB15" s="474" t="n"/>
+      <c r="BC15" s="474" t="n"/>
+      <c r="BD15" s="479" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1" s="264">
-      <c r="A16" s="479" t="n">
-        <v>7</v>
-      </c>
-      <c r="B16" s="480" t="n"/>
-      <c r="C16" s="480" t="n"/>
-      <c r="D16" s="481" t="n"/>
-      <c r="E16" s="482" t="n"/>
-      <c r="F16" s="480" t="n"/>
-      <c r="G16" s="480" t="n"/>
-      <c r="H16" s="480" t="n"/>
+      <c r="A16" s="497" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="481" t="n"/>
+      <c r="C16" s="482" t="n"/>
+      <c r="D16" s="498" t="n"/>
+      <c r="E16" s="481" t="n"/>
+      <c r="F16" s="481" t="n"/>
+      <c r="G16" s="482" t="n"/>
+      <c r="H16" s="498" t="n"/>
       <c r="I16" s="481" t="n"/>
-      <c r="J16" s="482" t="n"/>
-      <c r="K16" s="480" t="n"/>
-      <c r="L16" s="480" t="n"/>
-      <c r="M16" s="480" t="n"/>
-      <c r="N16" s="480" t="n"/>
-      <c r="O16" s="480" t="n"/>
-      <c r="P16" s="480" t="n"/>
-      <c r="Q16" s="480" t="n"/>
-      <c r="R16" s="480" t="n"/>
-      <c r="S16" s="480" t="n"/>
-      <c r="T16" s="480" t="n"/>
-      <c r="U16" s="480" t="n"/>
+      <c r="J16" s="481" t="n"/>
+      <c r="K16" s="481" t="n"/>
+      <c r="L16" s="481" t="n"/>
+      <c r="M16" s="481" t="n"/>
+      <c r="N16" s="481" t="n"/>
+      <c r="O16" s="481" t="n"/>
+      <c r="P16" s="481" t="n"/>
+      <c r="Q16" s="481" t="n"/>
+      <c r="R16" s="481" t="n"/>
+      <c r="S16" s="481" t="n"/>
+      <c r="T16" s="482" t="n"/>
+      <c r="U16" s="498" t="n"/>
       <c r="V16" s="481" t="n"/>
-      <c r="W16" s="482" t="n"/>
-      <c r="X16" s="480" t="n"/>
-      <c r="Y16" s="480" t="n"/>
-      <c r="Z16" s="480" t="n"/>
-      <c r="AA16" s="480" t="n"/>
-      <c r="AB16" s="480" t="n"/>
-      <c r="AC16" s="480" t="n"/>
-      <c r="AD16" s="480" t="n"/>
-      <c r="AE16" s="480" t="n"/>
-      <c r="AF16" s="480" t="n"/>
+      <c r="W16" s="481" t="n"/>
+      <c r="X16" s="481" t="n"/>
+      <c r="Y16" s="481" t="n"/>
+      <c r="Z16" s="481" t="n"/>
+      <c r="AA16" s="481" t="n"/>
+      <c r="AB16" s="481" t="n"/>
+      <c r="AC16" s="481" t="n"/>
+      <c r="AD16" s="482" t="n"/>
+      <c r="AE16" s="498" t="n"/>
+      <c r="AF16" s="481" t="n"/>
       <c r="AG16" s="481" t="n"/>
-      <c r="AH16" s="482" t="n"/>
-      <c r="AI16" s="480" t="n"/>
-      <c r="AJ16" s="480" t="n"/>
-      <c r="AK16" s="480" t="n"/>
+      <c r="AH16" s="481" t="n"/>
+      <c r="AI16" s="482" t="n"/>
+      <c r="AJ16" s="498" t="n"/>
+      <c r="AK16" s="481" t="n"/>
       <c r="AL16" s="481" t="n"/>
-      <c r="AM16" s="482" t="n"/>
-      <c r="AN16" s="480" t="n"/>
-      <c r="AO16" s="480" t="n"/>
-      <c r="AP16" s="480" t="n"/>
-      <c r="AQ16" s="480" t="n"/>
-      <c r="AR16" s="480" t="n"/>
-      <c r="AS16" s="480" t="n"/>
-      <c r="AT16" s="480" t="n"/>
+      <c r="AM16" s="481" t="n"/>
+      <c r="AN16" s="481" t="n"/>
+      <c r="AO16" s="481" t="n"/>
+      <c r="AP16" s="481" t="n"/>
+      <c r="AQ16" s="481" t="n"/>
+      <c r="AR16" s="482" t="n"/>
+      <c r="AS16" s="498" t="n"/>
+      <c r="AT16" s="481" t="n"/>
       <c r="AU16" s="481" t="n"/>
-      <c r="AV16" s="482" t="n"/>
-      <c r="AW16" s="480" t="n"/>
-      <c r="AX16" s="480" t="n"/>
-      <c r="AY16" s="480" t="n"/>
+      <c r="AV16" s="481" t="n"/>
+      <c r="AW16" s="481" t="n"/>
+      <c r="AX16" s="482" t="n"/>
+      <c r="AY16" s="499" t="n"/>
       <c r="AZ16" s="481" t="n"/>
-      <c r="BA16" s="483" t="n"/>
-      <c r="BB16" s="480" t="n"/>
-      <c r="BC16" s="480" t="n"/>
-      <c r="BD16" s="484" t="n"/>
+      <c r="BA16" s="481" t="n"/>
+      <c r="BB16" s="481" t="n"/>
+      <c r="BC16" s="481" t="n"/>
+      <c r="BD16" s="486" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1" s="264">
-      <c r="A17" s="479" t="n">
-        <v>8</v>
-      </c>
-      <c r="B17" s="480" t="n"/>
-      <c r="C17" s="480" t="n"/>
-      <c r="D17" s="481" t="n"/>
-      <c r="E17" s="485" t="n"/>
-      <c r="F17" s="480" t="n"/>
-      <c r="G17" s="480" t="n"/>
-      <c r="H17" s="480" t="n"/>
+      <c r="A17" s="497" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="481" t="n"/>
+      <c r="C17" s="482" t="n"/>
+      <c r="D17" s="500" t="n"/>
+      <c r="E17" s="481" t="n"/>
+      <c r="F17" s="481" t="n"/>
+      <c r="G17" s="482" t="n"/>
+      <c r="H17" s="500" t="n"/>
       <c r="I17" s="481" t="n"/>
-      <c r="J17" s="485" t="n"/>
-      <c r="K17" s="480" t="n"/>
-      <c r="L17" s="480" t="n"/>
-      <c r="M17" s="480" t="n"/>
-      <c r="N17" s="480" t="n"/>
-      <c r="O17" s="480" t="n"/>
-      <c r="P17" s="480" t="n"/>
-      <c r="Q17" s="480" t="n"/>
-      <c r="R17" s="480" t="n"/>
-      <c r="S17" s="480" t="n"/>
-      <c r="T17" s="480" t="n"/>
-      <c r="U17" s="480" t="n"/>
+      <c r="J17" s="481" t="n"/>
+      <c r="K17" s="481" t="n"/>
+      <c r="L17" s="481" t="n"/>
+      <c r="M17" s="481" t="n"/>
+      <c r="N17" s="481" t="n"/>
+      <c r="O17" s="481" t="n"/>
+      <c r="P17" s="481" t="n"/>
+      <c r="Q17" s="481" t="n"/>
+      <c r="R17" s="481" t="n"/>
+      <c r="S17" s="481" t="n"/>
+      <c r="T17" s="482" t="n"/>
+      <c r="U17" s="500" t="n"/>
       <c r="V17" s="481" t="n"/>
-      <c r="W17" s="485" t="n"/>
-      <c r="X17" s="480" t="n"/>
-      <c r="Y17" s="480" t="n"/>
-      <c r="Z17" s="480" t="n"/>
-      <c r="AA17" s="480" t="n"/>
-      <c r="AB17" s="480" t="n"/>
-      <c r="AC17" s="480" t="n"/>
-      <c r="AD17" s="480" t="n"/>
-      <c r="AE17" s="480" t="n"/>
-      <c r="AF17" s="480" t="n"/>
+      <c r="W17" s="481" t="n"/>
+      <c r="X17" s="481" t="n"/>
+      <c r="Y17" s="481" t="n"/>
+      <c r="Z17" s="481" t="n"/>
+      <c r="AA17" s="481" t="n"/>
+      <c r="AB17" s="481" t="n"/>
+      <c r="AC17" s="481" t="n"/>
+      <c r="AD17" s="482" t="n"/>
+      <c r="AE17" s="500" t="n"/>
+      <c r="AF17" s="481" t="n"/>
       <c r="AG17" s="481" t="n"/>
-      <c r="AH17" s="485" t="n"/>
-      <c r="AI17" s="480" t="n"/>
-      <c r="AJ17" s="480" t="n"/>
-      <c r="AK17" s="480" t="n"/>
+      <c r="AH17" s="481" t="n"/>
+      <c r="AI17" s="482" t="n"/>
+      <c r="AJ17" s="500" t="n"/>
+      <c r="AK17" s="481" t="n"/>
       <c r="AL17" s="481" t="n"/>
-      <c r="AM17" s="485" t="n"/>
-      <c r="AN17" s="480" t="n"/>
-      <c r="AO17" s="480" t="n"/>
-      <c r="AP17" s="480" t="n"/>
-      <c r="AQ17" s="480" t="n"/>
-      <c r="AR17" s="480" t="n"/>
-      <c r="AS17" s="480" t="n"/>
-      <c r="AT17" s="480" t="n"/>
+      <c r="AM17" s="481" t="n"/>
+      <c r="AN17" s="481" t="n"/>
+      <c r="AO17" s="481" t="n"/>
+      <c r="AP17" s="481" t="n"/>
+      <c r="AQ17" s="481" t="n"/>
+      <c r="AR17" s="482" t="n"/>
+      <c r="AS17" s="500" t="n"/>
+      <c r="AT17" s="481" t="n"/>
       <c r="AU17" s="481" t="n"/>
-      <c r="AV17" s="485" t="n"/>
-      <c r="AW17" s="480" t="n"/>
-      <c r="AX17" s="480" t="n"/>
-      <c r="AY17" s="480" t="n"/>
+      <c r="AV17" s="481" t="n"/>
+      <c r="AW17" s="481" t="n"/>
+      <c r="AX17" s="482" t="n"/>
+      <c r="AY17" s="501" t="n"/>
       <c r="AZ17" s="481" t="n"/>
-      <c r="BA17" s="486" t="n"/>
-      <c r="BB17" s="480" t="n"/>
-      <c r="BC17" s="480" t="n"/>
-      <c r="BD17" s="484" t="n"/>
+      <c r="BA17" s="481" t="n"/>
+      <c r="BB17" s="481" t="n"/>
+      <c r="BC17" s="481" t="n"/>
+      <c r="BD17" s="486" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1" s="264">
-      <c r="A18" s="479" t="n">
-        <v>9</v>
-      </c>
-      <c r="B18" s="480" t="n"/>
-      <c r="C18" s="480" t="n"/>
-      <c r="D18" s="481" t="n"/>
-      <c r="E18" s="482" t="n"/>
-      <c r="F18" s="480" t="n"/>
-      <c r="G18" s="480" t="n"/>
-      <c r="H18" s="480" t="n"/>
+      <c r="A18" s="497" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="481" t="n"/>
+      <c r="C18" s="482" t="n"/>
+      <c r="D18" s="498" t="n"/>
+      <c r="E18" s="481" t="n"/>
+      <c r="F18" s="481" t="n"/>
+      <c r="G18" s="482" t="n"/>
+      <c r="H18" s="498" t="n"/>
       <c r="I18" s="481" t="n"/>
-      <c r="J18" s="482" t="n"/>
-      <c r="K18" s="480" t="n"/>
-      <c r="L18" s="480" t="n"/>
-      <c r="M18" s="480" t="n"/>
-      <c r="N18" s="480" t="n"/>
-      <c r="O18" s="480" t="n"/>
-      <c r="P18" s="480" t="n"/>
-      <c r="Q18" s="480" t="n"/>
-      <c r="R18" s="480" t="n"/>
-      <c r="S18" s="480" t="n"/>
-      <c r="T18" s="480" t="n"/>
-      <c r="U18" s="480" t="n"/>
+      <c r="J18" s="481" t="n"/>
+      <c r="K18" s="481" t="n"/>
+      <c r="L18" s="481" t="n"/>
+      <c r="M18" s="481" t="n"/>
+      <c r="N18" s="481" t="n"/>
+      <c r="O18" s="481" t="n"/>
+      <c r="P18" s="481" t="n"/>
+      <c r="Q18" s="481" t="n"/>
+      <c r="R18" s="481" t="n"/>
+      <c r="S18" s="481" t="n"/>
+      <c r="T18" s="482" t="n"/>
+      <c r="U18" s="498" t="n"/>
       <c r="V18" s="481" t="n"/>
-      <c r="W18" s="482" t="n"/>
-      <c r="X18" s="480" t="n"/>
-      <c r="Y18" s="480" t="n"/>
-      <c r="Z18" s="480" t="n"/>
-      <c r="AA18" s="480" t="n"/>
-      <c r="AB18" s="480" t="n"/>
-      <c r="AC18" s="480" t="n"/>
-      <c r="AD18" s="480" t="n"/>
-      <c r="AE18" s="480" t="n"/>
-      <c r="AF18" s="480" t="n"/>
+      <c r="W18" s="481" t="n"/>
+      <c r="X18" s="481" t="n"/>
+      <c r="Y18" s="481" t="n"/>
+      <c r="Z18" s="481" t="n"/>
+      <c r="AA18" s="481" t="n"/>
+      <c r="AB18" s="481" t="n"/>
+      <c r="AC18" s="481" t="n"/>
+      <c r="AD18" s="482" t="n"/>
+      <c r="AE18" s="498" t="n"/>
+      <c r="AF18" s="481" t="n"/>
       <c r="AG18" s="481" t="n"/>
-      <c r="AH18" s="482" t="n"/>
-      <c r="AI18" s="480" t="n"/>
-      <c r="AJ18" s="480" t="n"/>
-      <c r="AK18" s="480" t="n"/>
+      <c r="AH18" s="481" t="n"/>
+      <c r="AI18" s="482" t="n"/>
+      <c r="AJ18" s="498" t="n"/>
+      <c r="AK18" s="481" t="n"/>
       <c r="AL18" s="481" t="n"/>
-      <c r="AM18" s="482" t="n"/>
-      <c r="AN18" s="480" t="n"/>
-      <c r="AO18" s="480" t="n"/>
-      <c r="AP18" s="480" t="n"/>
-      <c r="AQ18" s="480" t="n"/>
-      <c r="AR18" s="480" t="n"/>
-      <c r="AS18" s="480" t="n"/>
-      <c r="AT18" s="480" t="n"/>
+      <c r="AM18" s="481" t="n"/>
+      <c r="AN18" s="481" t="n"/>
+      <c r="AO18" s="481" t="n"/>
+      <c r="AP18" s="481" t="n"/>
+      <c r="AQ18" s="481" t="n"/>
+      <c r="AR18" s="482" t="n"/>
+      <c r="AS18" s="498" t="n"/>
+      <c r="AT18" s="481" t="n"/>
       <c r="AU18" s="481" t="n"/>
-      <c r="AV18" s="482" t="n"/>
-      <c r="AW18" s="480" t="n"/>
-      <c r="AX18" s="480" t="n"/>
-      <c r="AY18" s="480" t="n"/>
+      <c r="AV18" s="481" t="n"/>
+      <c r="AW18" s="481" t="n"/>
+      <c r="AX18" s="482" t="n"/>
+      <c r="AY18" s="499" t="n"/>
       <c r="AZ18" s="481" t="n"/>
-      <c r="BA18" s="483" t="n"/>
-      <c r="BB18" s="480" t="n"/>
-      <c r="BC18" s="480" t="n"/>
-      <c r="BD18" s="484" t="n"/>
+      <c r="BA18" s="481" t="n"/>
+      <c r="BB18" s="481" t="n"/>
+      <c r="BC18" s="481" t="n"/>
+      <c r="BD18" s="486" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1" s="264">
-      <c r="A19" s="479" t="n">
-        <v>10</v>
-      </c>
-      <c r="B19" s="480" t="n"/>
-      <c r="C19" s="480" t="n"/>
-      <c r="D19" s="481" t="n"/>
-      <c r="E19" s="485" t="n"/>
-      <c r="F19" s="480" t="n"/>
-      <c r="G19" s="480" t="n"/>
-      <c r="H19" s="480" t="n"/>
+      <c r="A19" s="497" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="481" t="n"/>
+      <c r="C19" s="482" t="n"/>
+      <c r="D19" s="500" t="n"/>
+      <c r="E19" s="481" t="n"/>
+      <c r="F19" s="481" t="n"/>
+      <c r="G19" s="482" t="n"/>
+      <c r="H19" s="500" t="n"/>
       <c r="I19" s="481" t="n"/>
-      <c r="J19" s="485" t="n"/>
-      <c r="K19" s="480" t="n"/>
-      <c r="L19" s="480" t="n"/>
-      <c r="M19" s="480" t="n"/>
-      <c r="N19" s="480" t="n"/>
-      <c r="O19" s="480" t="n"/>
-      <c r="P19" s="480" t="n"/>
-      <c r="Q19" s="480" t="n"/>
-      <c r="R19" s="480" t="n"/>
-      <c r="S19" s="480" t="n"/>
-      <c r="T19" s="480" t="n"/>
-      <c r="U19" s="480" t="n"/>
+      <c r="J19" s="481" t="n"/>
+      <c r="K19" s="481" t="n"/>
+      <c r="L19" s="481" t="n"/>
+      <c r="M19" s="481" t="n"/>
+      <c r="N19" s="481" t="n"/>
+      <c r="O19" s="481" t="n"/>
+      <c r="P19" s="481" t="n"/>
+      <c r="Q19" s="481" t="n"/>
+      <c r="R19" s="481" t="n"/>
+      <c r="S19" s="481" t="n"/>
+      <c r="T19" s="482" t="n"/>
+      <c r="U19" s="500" t="n"/>
       <c r="V19" s="481" t="n"/>
-      <c r="W19" s="485" t="n"/>
-      <c r="X19" s="480" t="n"/>
-      <c r="Y19" s="480" t="n"/>
-      <c r="Z19" s="480" t="n"/>
-      <c r="AA19" s="480" t="n"/>
-      <c r="AB19" s="480" t="n"/>
-      <c r="AC19" s="480" t="n"/>
-      <c r="AD19" s="480" t="n"/>
-      <c r="AE19" s="480" t="n"/>
-      <c r="AF19" s="480" t="n"/>
+      <c r="W19" s="481" t="n"/>
+      <c r="X19" s="481" t="n"/>
+      <c r="Y19" s="481" t="n"/>
+      <c r="Z19" s="481" t="n"/>
+      <c r="AA19" s="481" t="n"/>
+      <c r="AB19" s="481" t="n"/>
+      <c r="AC19" s="481" t="n"/>
+      <c r="AD19" s="482" t="n"/>
+      <c r="AE19" s="500" t="n"/>
+      <c r="AF19" s="481" t="n"/>
       <c r="AG19" s="481" t="n"/>
-      <c r="AH19" s="485" t="n"/>
-      <c r="AI19" s="480" t="n"/>
-      <c r="AJ19" s="480" t="n"/>
-      <c r="AK19" s="480" t="n"/>
+      <c r="AH19" s="481" t="n"/>
+      <c r="AI19" s="482" t="n"/>
+      <c r="AJ19" s="500" t="n"/>
+      <c r="AK19" s="481" t="n"/>
       <c r="AL19" s="481" t="n"/>
-      <c r="AM19" s="485" t="n"/>
-      <c r="AN19" s="480" t="n"/>
-      <c r="AO19" s="480" t="n"/>
-      <c r="AP19" s="480" t="n"/>
-      <c r="AQ19" s="480" t="n"/>
-      <c r="AR19" s="480" t="n"/>
-      <c r="AS19" s="480" t="n"/>
-      <c r="AT19" s="480" t="n"/>
+      <c r="AM19" s="481" t="n"/>
+      <c r="AN19" s="481" t="n"/>
+      <c r="AO19" s="481" t="n"/>
+      <c r="AP19" s="481" t="n"/>
+      <c r="AQ19" s="481" t="n"/>
+      <c r="AR19" s="482" t="n"/>
+      <c r="AS19" s="500" t="n"/>
+      <c r="AT19" s="481" t="n"/>
       <c r="AU19" s="481" t="n"/>
-      <c r="AV19" s="485" t="n"/>
-      <c r="AW19" s="480" t="n"/>
-      <c r="AX19" s="480" t="n"/>
-      <c r="AY19" s="480" t="n"/>
+      <c r="AV19" s="481" t="n"/>
+      <c r="AW19" s="481" t="n"/>
+      <c r="AX19" s="482" t="n"/>
+      <c r="AY19" s="501" t="n"/>
       <c r="AZ19" s="481" t="n"/>
-      <c r="BA19" s="486" t="n"/>
-      <c r="BB19" s="480" t="n"/>
-      <c r="BC19" s="480" t="n"/>
-      <c r="BD19" s="484" t="n"/>
+      <c r="BA19" s="481" t="n"/>
+      <c r="BB19" s="481" t="n"/>
+      <c r="BC19" s="481" t="n"/>
+      <c r="BD19" s="486" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1" s="264">
-      <c r="A20" s="479" t="n">
-        <v>11</v>
-      </c>
-      <c r="B20" s="480" t="n"/>
-      <c r="C20" s="480" t="n"/>
-      <c r="D20" s="481" t="n"/>
-      <c r="E20" s="482" t="n"/>
-      <c r="F20" s="480" t="n"/>
-      <c r="G20" s="480" t="n"/>
-      <c r="H20" s="480" t="n"/>
+      <c r="A20" s="497" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="481" t="n"/>
+      <c r="C20" s="482" t="n"/>
+      <c r="D20" s="498" t="n"/>
+      <c r="E20" s="481" t="n"/>
+      <c r="F20" s="481" t="n"/>
+      <c r="G20" s="482" t="n"/>
+      <c r="H20" s="498" t="n"/>
       <c r="I20" s="481" t="n"/>
-      <c r="J20" s="482" t="n"/>
-      <c r="K20" s="480" t="n"/>
-      <c r="L20" s="480" t="n"/>
-      <c r="M20" s="480" t="n"/>
-      <c r="N20" s="480" t="n"/>
-      <c r="O20" s="480" t="n"/>
-      <c r="P20" s="480" t="n"/>
-      <c r="Q20" s="480" t="n"/>
-      <c r="R20" s="480" t="n"/>
-      <c r="S20" s="480" t="n"/>
-      <c r="T20" s="480" t="n"/>
-      <c r="U20" s="480" t="n"/>
+      <c r="J20" s="481" t="n"/>
+      <c r="K20" s="481" t="n"/>
+      <c r="L20" s="481" t="n"/>
+      <c r="M20" s="481" t="n"/>
+      <c r="N20" s="481" t="n"/>
+      <c r="O20" s="481" t="n"/>
+      <c r="P20" s="481" t="n"/>
+      <c r="Q20" s="481" t="n"/>
+      <c r="R20" s="481" t="n"/>
+      <c r="S20" s="481" t="n"/>
+      <c r="T20" s="482" t="n"/>
+      <c r="U20" s="498" t="n"/>
       <c r="V20" s="481" t="n"/>
-      <c r="W20" s="482" t="n"/>
-      <c r="X20" s="480" t="n"/>
-      <c r="Y20" s="480" t="n"/>
-      <c r="Z20" s="480" t="n"/>
-      <c r="AA20" s="480" t="n"/>
-      <c r="AB20" s="480" t="n"/>
-      <c r="AC20" s="480" t="n"/>
-      <c r="AD20" s="480" t="n"/>
-      <c r="AE20" s="480" t="n"/>
-      <c r="AF20" s="480" t="n"/>
+      <c r="W20" s="481" t="n"/>
+      <c r="X20" s="481" t="n"/>
+      <c r="Y20" s="481" t="n"/>
+      <c r="Z20" s="481" t="n"/>
+      <c r="AA20" s="481" t="n"/>
+      <c r="AB20" s="481" t="n"/>
+      <c r="AC20" s="481" t="n"/>
+      <c r="AD20" s="482" t="n"/>
+      <c r="AE20" s="498" t="n"/>
+      <c r="AF20" s="481" t="n"/>
       <c r="AG20" s="481" t="n"/>
-      <c r="AH20" s="482" t="n"/>
-      <c r="AI20" s="480" t="n"/>
-      <c r="AJ20" s="480" t="n"/>
-      <c r="AK20" s="480" t="n"/>
+      <c r="AH20" s="481" t="n"/>
+      <c r="AI20" s="482" t="n"/>
+      <c r="AJ20" s="498" t="n"/>
+      <c r="AK20" s="481" t="n"/>
       <c r="AL20" s="481" t="n"/>
-      <c r="AM20" s="482" t="n"/>
-      <c r="AN20" s="480" t="n"/>
-      <c r="AO20" s="480" t="n"/>
-      <c r="AP20" s="480" t="n"/>
-      <c r="AQ20" s="480" t="n"/>
-      <c r="AR20" s="480" t="n"/>
-      <c r="AS20" s="480" t="n"/>
-      <c r="AT20" s="480" t="n"/>
+      <c r="AM20" s="481" t="n"/>
+      <c r="AN20" s="481" t="n"/>
+      <c r="AO20" s="481" t="n"/>
+      <c r="AP20" s="481" t="n"/>
+      <c r="AQ20" s="481" t="n"/>
+      <c r="AR20" s="482" t="n"/>
+      <c r="AS20" s="498" t="n"/>
+      <c r="AT20" s="481" t="n"/>
       <c r="AU20" s="481" t="n"/>
-      <c r="AV20" s="482" t="n"/>
-      <c r="AW20" s="480" t="n"/>
-      <c r="AX20" s="480" t="n"/>
-      <c r="AY20" s="480" t="n"/>
+      <c r="AV20" s="481" t="n"/>
+      <c r="AW20" s="481" t="n"/>
+      <c r="AX20" s="482" t="n"/>
+      <c r="AY20" s="499" t="n"/>
       <c r="AZ20" s="481" t="n"/>
-      <c r="BA20" s="483" t="n"/>
-      <c r="BB20" s="480" t="n"/>
-      <c r="BC20" s="480" t="n"/>
-      <c r="BD20" s="484" t="n"/>
+      <c r="BA20" s="481" t="n"/>
+      <c r="BB20" s="481" t="n"/>
+      <c r="BC20" s="481" t="n"/>
+      <c r="BD20" s="486" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1" s="264">
-      <c r="A21" s="479" t="n">
-        <v>12</v>
-      </c>
-      <c r="B21" s="480" t="n"/>
-      <c r="C21" s="480" t="n"/>
-      <c r="D21" s="481" t="n"/>
-      <c r="E21" s="485" t="n"/>
-      <c r="F21" s="480" t="n"/>
-      <c r="G21" s="480" t="n"/>
-      <c r="H21" s="480" t="n"/>
+      <c r="A21" s="497" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="481" t="n"/>
+      <c r="C21" s="482" t="n"/>
+      <c r="D21" s="500" t="n"/>
+      <c r="E21" s="481" t="n"/>
+      <c r="F21" s="481" t="n"/>
+      <c r="G21" s="482" t="n"/>
+      <c r="H21" s="500" t="n"/>
       <c r="I21" s="481" t="n"/>
-      <c r="J21" s="485" t="n"/>
-      <c r="K21" s="480" t="n"/>
-      <c r="L21" s="480" t="n"/>
-      <c r="M21" s="480" t="n"/>
-      <c r="N21" s="480" t="n"/>
-      <c r="O21" s="480" t="n"/>
-      <c r="P21" s="480" t="n"/>
-      <c r="Q21" s="480" t="n"/>
-      <c r="R21" s="480" t="n"/>
-      <c r="S21" s="480" t="n"/>
-      <c r="T21" s="480" t="n"/>
-      <c r="U21" s="480" t="n"/>
+      <c r="J21" s="481" t="n"/>
+      <c r="K21" s="481" t="n"/>
+      <c r="L21" s="481" t="n"/>
+      <c r="M21" s="481" t="n"/>
+      <c r="N21" s="481" t="n"/>
+      <c r="O21" s="481" t="n"/>
+      <c r="P21" s="481" t="n"/>
+      <c r="Q21" s="481" t="n"/>
+      <c r="R21" s="481" t="n"/>
+      <c r="S21" s="481" t="n"/>
+      <c r="T21" s="482" t="n"/>
+      <c r="U21" s="500" t="n"/>
       <c r="V21" s="481" t="n"/>
-      <c r="W21" s="485" t="n"/>
-      <c r="X21" s="480" t="n"/>
-      <c r="Y21" s="480" t="n"/>
-      <c r="Z21" s="480" t="n"/>
-      <c r="AA21" s="480" t="n"/>
-      <c r="AB21" s="480" t="n"/>
-      <c r="AC21" s="480" t="n"/>
-      <c r="AD21" s="480" t="n"/>
-      <c r="AE21" s="480" t="n"/>
-      <c r="AF21" s="480" t="n"/>
+      <c r="W21" s="481" t="n"/>
+      <c r="X21" s="481" t="n"/>
+      <c r="Y21" s="481" t="n"/>
+      <c r="Z21" s="481" t="n"/>
+      <c r="AA21" s="481" t="n"/>
+      <c r="AB21" s="481" t="n"/>
+      <c r="AC21" s="481" t="n"/>
+      <c r="AD21" s="482" t="n"/>
+      <c r="AE21" s="500" t="n"/>
+      <c r="AF21" s="481" t="n"/>
       <c r="AG21" s="481" t="n"/>
-      <c r="AH21" s="485" t="n"/>
-      <c r="AI21" s="480" t="n"/>
-      <c r="AJ21" s="480" t="n"/>
-      <c r="AK21" s="480" t="n"/>
+      <c r="AH21" s="481" t="n"/>
+      <c r="AI21" s="482" t="n"/>
+      <c r="AJ21" s="500" t="n"/>
+      <c r="AK21" s="481" t="n"/>
       <c r="AL21" s="481" t="n"/>
-      <c r="AM21" s="485" t="n"/>
-      <c r="AN21" s="480" t="n"/>
-      <c r="AO21" s="480" t="n"/>
-      <c r="AP21" s="480" t="n"/>
-      <c r="AQ21" s="480" t="n"/>
-      <c r="AR21" s="480" t="n"/>
-      <c r="AS21" s="480" t="n"/>
-      <c r="AT21" s="480" t="n"/>
+      <c r="AM21" s="481" t="n"/>
+      <c r="AN21" s="481" t="n"/>
+      <c r="AO21" s="481" t="n"/>
+      <c r="AP21" s="481" t="n"/>
+      <c r="AQ21" s="481" t="n"/>
+      <c r="AR21" s="482" t="n"/>
+      <c r="AS21" s="500" t="n"/>
+      <c r="AT21" s="481" t="n"/>
       <c r="AU21" s="481" t="n"/>
-      <c r="AV21" s="485" t="n"/>
-      <c r="AW21" s="480" t="n"/>
-      <c r="AX21" s="480" t="n"/>
-      <c r="AY21" s="480" t="n"/>
+      <c r="AV21" s="481" t="n"/>
+      <c r="AW21" s="481" t="n"/>
+      <c r="AX21" s="482" t="n"/>
+      <c r="AY21" s="501" t="n"/>
       <c r="AZ21" s="481" t="n"/>
-      <c r="BA21" s="486" t="n"/>
-      <c r="BB21" s="480" t="n"/>
-      <c r="BC21" s="480" t="n"/>
-      <c r="BD21" s="484" t="n"/>
+      <c r="BA21" s="481" t="n"/>
+      <c r="BB21" s="481" t="n"/>
+      <c r="BC21" s="481" t="n"/>
+      <c r="BD21" s="486" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1" s="264">
-      <c r="A22" s="479" t="n">
-        <v>13</v>
-      </c>
-      <c r="B22" s="480" t="n"/>
-      <c r="C22" s="480" t="n"/>
-      <c r="D22" s="481" t="n"/>
-      <c r="E22" s="482" t="n"/>
-      <c r="F22" s="480" t="n"/>
-      <c r="G22" s="480" t="n"/>
-      <c r="H22" s="480" t="n"/>
+      <c r="A22" s="497" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="481" t="n"/>
+      <c r="C22" s="482" t="n"/>
+      <c r="D22" s="498" t="n"/>
+      <c r="E22" s="481" t="n"/>
+      <c r="F22" s="481" t="n"/>
+      <c r="G22" s="482" t="n"/>
+      <c r="H22" s="498" t="n"/>
       <c r="I22" s="481" t="n"/>
-      <c r="J22" s="482" t="n"/>
-      <c r="K22" s="480" t="n"/>
-      <c r="L22" s="480" t="n"/>
-      <c r="M22" s="480" t="n"/>
-      <c r="N22" s="480" t="n"/>
-      <c r="O22" s="480" t="n"/>
-      <c r="P22" s="480" t="n"/>
-      <c r="Q22" s="480" t="n"/>
-      <c r="R22" s="480" t="n"/>
-      <c r="S22" s="480" t="n"/>
-      <c r="T22" s="480" t="n"/>
-      <c r="U22" s="480" t="n"/>
+      <c r="J22" s="481" t="n"/>
+      <c r="K22" s="481" t="n"/>
+      <c r="L22" s="481" t="n"/>
+      <c r="M22" s="481" t="n"/>
+      <c r="N22" s="481" t="n"/>
+      <c r="O22" s="481" t="n"/>
+      <c r="P22" s="481" t="n"/>
+      <c r="Q22" s="481" t="n"/>
+      <c r="R22" s="481" t="n"/>
+      <c r="S22" s="481" t="n"/>
+      <c r="T22" s="482" t="n"/>
+      <c r="U22" s="498" t="n"/>
       <c r="V22" s="481" t="n"/>
-      <c r="W22" s="482" t="n"/>
-      <c r="X22" s="480" t="n"/>
-      <c r="Y22" s="480" t="n"/>
-      <c r="Z22" s="480" t="n"/>
-      <c r="AA22" s="480" t="n"/>
-      <c r="AB22" s="480" t="n"/>
-      <c r="AC22" s="480" t="n"/>
-      <c r="AD22" s="480" t="n"/>
-      <c r="AE22" s="480" t="n"/>
-      <c r="AF22" s="480" t="n"/>
+      <c r="W22" s="481" t="n"/>
+      <c r="X22" s="481" t="n"/>
+      <c r="Y22" s="481" t="n"/>
+      <c r="Z22" s="481" t="n"/>
+      <c r="AA22" s="481" t="n"/>
+      <c r="AB22" s="481" t="n"/>
+      <c r="AC22" s="481" t="n"/>
+      <c r="AD22" s="482" t="n"/>
+      <c r="AE22" s="498" t="n"/>
+      <c r="AF22" s="481" t="n"/>
       <c r="AG22" s="481" t="n"/>
-      <c r="AH22" s="482" t="n"/>
-      <c r="AI22" s="480" t="n"/>
-      <c r="AJ22" s="480" t="n"/>
-      <c r="AK22" s="480" t="n"/>
+      <c r="AH22" s="481" t="n"/>
+      <c r="AI22" s="482" t="n"/>
+      <c r="AJ22" s="498" t="n"/>
+      <c r="AK22" s="481" t="n"/>
       <c r="AL22" s="481" t="n"/>
-      <c r="AM22" s="482" t="n"/>
-      <c r="AN22" s="480" t="n"/>
-      <c r="AO22" s="480" t="n"/>
-      <c r="AP22" s="480" t="n"/>
-      <c r="AQ22" s="480" t="n"/>
-      <c r="AR22" s="480" t="n"/>
-      <c r="AS22" s="480" t="n"/>
-      <c r="AT22" s="480" t="n"/>
+      <c r="AM22" s="481" t="n"/>
+      <c r="AN22" s="481" t="n"/>
+      <c r="AO22" s="481" t="n"/>
+      <c r="AP22" s="481" t="n"/>
+      <c r="AQ22" s="481" t="n"/>
+      <c r="AR22" s="482" t="n"/>
+      <c r="AS22" s="498" t="n"/>
+      <c r="AT22" s="481" t="n"/>
       <c r="AU22" s="481" t="n"/>
-      <c r="AV22" s="482" t="n"/>
-      <c r="AW22" s="480" t="n"/>
-      <c r="AX22" s="480" t="n"/>
-      <c r="AY22" s="480" t="n"/>
+      <c r="AV22" s="481" t="n"/>
+      <c r="AW22" s="481" t="n"/>
+      <c r="AX22" s="482" t="n"/>
+      <c r="AY22" s="499" t="n"/>
       <c r="AZ22" s="481" t="n"/>
-      <c r="BA22" s="483" t="n"/>
-      <c r="BB22" s="480" t="n"/>
-      <c r="BC22" s="480" t="n"/>
-      <c r="BD22" s="484" t="n"/>
+      <c r="BA22" s="481" t="n"/>
+      <c r="BB22" s="481" t="n"/>
+      <c r="BC22" s="481" t="n"/>
+      <c r="BD22" s="486" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1" s="264">
-      <c r="A23" s="479" t="n">
-        <v>14</v>
-      </c>
-      <c r="B23" s="480" t="n"/>
-      <c r="C23" s="480" t="n"/>
-      <c r="D23" s="481" t="n"/>
-      <c r="E23" s="485" t="n"/>
-      <c r="F23" s="480" t="n"/>
-      <c r="G23" s="480" t="n"/>
-      <c r="H23" s="480" t="n"/>
+      <c r="A23" s="497" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="481" t="n"/>
+      <c r="C23" s="482" t="n"/>
+      <c r="D23" s="500" t="n"/>
+      <c r="E23" s="481" t="n"/>
+      <c r="F23" s="481" t="n"/>
+      <c r="G23" s="482" t="n"/>
+      <c r="H23" s="500" t="n"/>
       <c r="I23" s="481" t="n"/>
-      <c r="J23" s="485" t="n"/>
-      <c r="K23" s="480" t="n"/>
-      <c r="L23" s="480" t="n"/>
-      <c r="M23" s="480" t="n"/>
-      <c r="N23" s="480" t="n"/>
-      <c r="O23" s="480" t="n"/>
-      <c r="P23" s="480" t="n"/>
-      <c r="Q23" s="480" t="n"/>
-      <c r="R23" s="480" t="n"/>
-      <c r="S23" s="480" t="n"/>
-      <c r="T23" s="480" t="n"/>
-      <c r="U23" s="480" t="n"/>
+      <c r="J23" s="481" t="n"/>
+      <c r="K23" s="481" t="n"/>
+      <c r="L23" s="481" t="n"/>
+      <c r="M23" s="481" t="n"/>
+      <c r="N23" s="481" t="n"/>
+      <c r="O23" s="481" t="n"/>
+      <c r="P23" s="481" t="n"/>
+      <c r="Q23" s="481" t="n"/>
+      <c r="R23" s="481" t="n"/>
+      <c r="S23" s="481" t="n"/>
+      <c r="T23" s="482" t="n"/>
+      <c r="U23" s="500" t="n"/>
       <c r="V23" s="481" t="n"/>
-      <c r="W23" s="485" t="n"/>
-      <c r="X23" s="480" t="n"/>
-      <c r="Y23" s="480" t="n"/>
-      <c r="Z23" s="480" t="n"/>
-      <c r="AA23" s="480" t="n"/>
-      <c r="AB23" s="480" t="n"/>
-      <c r="AC23" s="480" t="n"/>
-      <c r="AD23" s="480" t="n"/>
-      <c r="AE23" s="480" t="n"/>
-      <c r="AF23" s="480" t="n"/>
+      <c r="W23" s="481" t="n"/>
+      <c r="X23" s="481" t="n"/>
+      <c r="Y23" s="481" t="n"/>
+      <c r="Z23" s="481" t="n"/>
+      <c r="AA23" s="481" t="n"/>
+      <c r="AB23" s="481" t="n"/>
+      <c r="AC23" s="481" t="n"/>
+      <c r="AD23" s="482" t="n"/>
+      <c r="AE23" s="500" t="n"/>
+      <c r="AF23" s="481" t="n"/>
       <c r="AG23" s="481" t="n"/>
-      <c r="AH23" s="485" t="n"/>
-      <c r="AI23" s="480" t="n"/>
-      <c r="AJ23" s="480" t="n"/>
-      <c r="AK23" s="480" t="n"/>
+      <c r="AH23" s="481" t="n"/>
+      <c r="AI23" s="482" t="n"/>
+      <c r="AJ23" s="500" t="n"/>
+      <c r="AK23" s="481" t="n"/>
       <c r="AL23" s="481" t="n"/>
-      <c r="AM23" s="485" t="n"/>
-      <c r="AN23" s="480" t="n"/>
-      <c r="AO23" s="480" t="n"/>
-      <c r="AP23" s="480" t="n"/>
-      <c r="AQ23" s="480" t="n"/>
-      <c r="AR23" s="480" t="n"/>
-      <c r="AS23" s="480" t="n"/>
-      <c r="AT23" s="480" t="n"/>
+      <c r="AM23" s="481" t="n"/>
+      <c r="AN23" s="481" t="n"/>
+      <c r="AO23" s="481" t="n"/>
+      <c r="AP23" s="481" t="n"/>
+      <c r="AQ23" s="481" t="n"/>
+      <c r="AR23" s="482" t="n"/>
+      <c r="AS23" s="500" t="n"/>
+      <c r="AT23" s="481" t="n"/>
       <c r="AU23" s="481" t="n"/>
-      <c r="AV23" s="485" t="n"/>
-      <c r="AW23" s="480" t="n"/>
-      <c r="AX23" s="480" t="n"/>
-      <c r="AY23" s="480" t="n"/>
+      <c r="AV23" s="481" t="n"/>
+      <c r="AW23" s="481" t="n"/>
+      <c r="AX23" s="482" t="n"/>
+      <c r="AY23" s="501" t="n"/>
       <c r="AZ23" s="481" t="n"/>
-      <c r="BA23" s="486" t="n"/>
-      <c r="BB23" s="480" t="n"/>
-      <c r="BC23" s="480" t="n"/>
-      <c r="BD23" s="484" t="n"/>
+      <c r="BA23" s="481" t="n"/>
+      <c r="BB23" s="481" t="n"/>
+      <c r="BC23" s="481" t="n"/>
+      <c r="BD23" s="486" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1" s="264">
-      <c r="A24" s="479" t="n">
-        <v>15</v>
-      </c>
-      <c r="B24" s="480" t="n"/>
-      <c r="C24" s="480" t="n"/>
-      <c r="D24" s="481" t="n"/>
-      <c r="E24" s="482" t="n"/>
-      <c r="F24" s="480" t="n"/>
-      <c r="G24" s="480" t="n"/>
-      <c r="H24" s="480" t="n"/>
+      <c r="A24" s="497" t="n">
+        <v>9</v>
+      </c>
+      <c r="B24" s="481" t="n"/>
+      <c r="C24" s="482" t="n"/>
+      <c r="D24" s="498" t="n"/>
+      <c r="E24" s="481" t="n"/>
+      <c r="F24" s="481" t="n"/>
+      <c r="G24" s="482" t="n"/>
+      <c r="H24" s="498" t="n"/>
       <c r="I24" s="481" t="n"/>
-      <c r="J24" s="482" t="n"/>
-      <c r="K24" s="480" t="n"/>
-      <c r="L24" s="480" t="n"/>
-      <c r="M24" s="480" t="n"/>
-      <c r="N24" s="480" t="n"/>
-      <c r="O24" s="480" t="n"/>
-      <c r="P24" s="480" t="n"/>
-      <c r="Q24" s="480" t="n"/>
-      <c r="R24" s="480" t="n"/>
-      <c r="S24" s="480" t="n"/>
-      <c r="T24" s="480" t="n"/>
-      <c r="U24" s="480" t="n"/>
+      <c r="J24" s="481" t="n"/>
+      <c r="K24" s="481" t="n"/>
+      <c r="L24" s="481" t="n"/>
+      <c r="M24" s="481" t="n"/>
+      <c r="N24" s="481" t="n"/>
+      <c r="O24" s="481" t="n"/>
+      <c r="P24" s="481" t="n"/>
+      <c r="Q24" s="481" t="n"/>
+      <c r="R24" s="481" t="n"/>
+      <c r="S24" s="481" t="n"/>
+      <c r="T24" s="482" t="n"/>
+      <c r="U24" s="498" t="n"/>
       <c r="V24" s="481" t="n"/>
-      <c r="W24" s="482" t="n"/>
-      <c r="X24" s="480" t="n"/>
-      <c r="Y24" s="480" t="n"/>
-      <c r="Z24" s="480" t="n"/>
-      <c r="AA24" s="480" t="n"/>
-      <c r="AB24" s="480" t="n"/>
-      <c r="AC24" s="480" t="n"/>
-      <c r="AD24" s="480" t="n"/>
-      <c r="AE24" s="480" t="n"/>
-      <c r="AF24" s="480" t="n"/>
+      <c r="W24" s="481" t="n"/>
+      <c r="X24" s="481" t="n"/>
+      <c r="Y24" s="481" t="n"/>
+      <c r="Z24" s="481" t="n"/>
+      <c r="AA24" s="481" t="n"/>
+      <c r="AB24" s="481" t="n"/>
+      <c r="AC24" s="481" t="n"/>
+      <c r="AD24" s="482" t="n"/>
+      <c r="AE24" s="498" t="n"/>
+      <c r="AF24" s="481" t="n"/>
       <c r="AG24" s="481" t="n"/>
-      <c r="AH24" s="482" t="n"/>
-      <c r="AI24" s="480" t="n"/>
-      <c r="AJ24" s="480" t="n"/>
-      <c r="AK24" s="480" t="n"/>
+      <c r="AH24" s="481" t="n"/>
+      <c r="AI24" s="482" t="n"/>
+      <c r="AJ24" s="498" t="n"/>
+      <c r="AK24" s="481" t="n"/>
       <c r="AL24" s="481" t="n"/>
-      <c r="AM24" s="482" t="n"/>
-      <c r="AN24" s="480" t="n"/>
-      <c r="AO24" s="480" t="n"/>
-      <c r="AP24" s="480" t="n"/>
-      <c r="AQ24" s="480" t="n"/>
-      <c r="AR24" s="480" t="n"/>
-      <c r="AS24" s="480" t="n"/>
-      <c r="AT24" s="480" t="n"/>
+      <c r="AM24" s="481" t="n"/>
+      <c r="AN24" s="481" t="n"/>
+      <c r="AO24" s="481" t="n"/>
+      <c r="AP24" s="481" t="n"/>
+      <c r="AQ24" s="481" t="n"/>
+      <c r="AR24" s="482" t="n"/>
+      <c r="AS24" s="498" t="n"/>
+      <c r="AT24" s="481" t="n"/>
       <c r="AU24" s="481" t="n"/>
-      <c r="AV24" s="482" t="n"/>
-      <c r="AW24" s="480" t="n"/>
-      <c r="AX24" s="480" t="n"/>
-      <c r="AY24" s="480" t="n"/>
+      <c r="AV24" s="481" t="n"/>
+      <c r="AW24" s="481" t="n"/>
+      <c r="AX24" s="482" t="n"/>
+      <c r="AY24" s="499" t="n"/>
       <c r="AZ24" s="481" t="n"/>
-      <c r="BA24" s="483" t="n"/>
-      <c r="BB24" s="480" t="n"/>
-      <c r="BC24" s="480" t="n"/>
-      <c r="BD24" s="484" t="n"/>
+      <c r="BA24" s="481" t="n"/>
+      <c r="BB24" s="481" t="n"/>
+      <c r="BC24" s="481" t="n"/>
+      <c r="BD24" s="486" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1" s="264">
-      <c r="A25" s="487" t="n">
+      <c r="A25" s="497" t="n">
+        <v>10</v>
+      </c>
+      <c r="B25" s="481" t="n"/>
+      <c r="C25" s="482" t="n"/>
+      <c r="D25" s="500" t="n"/>
+      <c r="E25" s="481" t="n"/>
+      <c r="F25" s="481" t="n"/>
+      <c r="G25" s="482" t="n"/>
+      <c r="H25" s="500" t="n"/>
+      <c r="I25" s="481" t="n"/>
+      <c r="J25" s="481" t="n"/>
+      <c r="K25" s="481" t="n"/>
+      <c r="L25" s="481" t="n"/>
+      <c r="M25" s="481" t="n"/>
+      <c r="N25" s="481" t="n"/>
+      <c r="O25" s="481" t="n"/>
+      <c r="P25" s="481" t="n"/>
+      <c r="Q25" s="481" t="n"/>
+      <c r="R25" s="481" t="n"/>
+      <c r="S25" s="481" t="n"/>
+      <c r="T25" s="482" t="n"/>
+      <c r="U25" s="500" t="n"/>
+      <c r="V25" s="481" t="n"/>
+      <c r="W25" s="481" t="n"/>
+      <c r="X25" s="481" t="n"/>
+      <c r="Y25" s="481" t="n"/>
+      <c r="Z25" s="481" t="n"/>
+      <c r="AA25" s="481" t="n"/>
+      <c r="AB25" s="481" t="n"/>
+      <c r="AC25" s="481" t="n"/>
+      <c r="AD25" s="482" t="n"/>
+      <c r="AE25" s="500" t="n"/>
+      <c r="AF25" s="481" t="n"/>
+      <c r="AG25" s="481" t="n"/>
+      <c r="AH25" s="481" t="n"/>
+      <c r="AI25" s="482" t="n"/>
+      <c r="AJ25" s="500" t="n"/>
+      <c r="AK25" s="481" t="n"/>
+      <c r="AL25" s="481" t="n"/>
+      <c r="AM25" s="481" t="n"/>
+      <c r="AN25" s="481" t="n"/>
+      <c r="AO25" s="481" t="n"/>
+      <c r="AP25" s="481" t="n"/>
+      <c r="AQ25" s="481" t="n"/>
+      <c r="AR25" s="482" t="n"/>
+      <c r="AS25" s="500" t="n"/>
+      <c r="AT25" s="481" t="n"/>
+      <c r="AU25" s="481" t="n"/>
+      <c r="AV25" s="481" t="n"/>
+      <c r="AW25" s="481" t="n"/>
+      <c r="AX25" s="482" t="n"/>
+      <c r="AY25" s="501" t="n"/>
+      <c r="AZ25" s="481" t="n"/>
+      <c r="BA25" s="481" t="n"/>
+      <c r="BB25" s="481" t="n"/>
+      <c r="BC25" s="481" t="n"/>
+      <c r="BD25" s="486" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" s="264">
+      <c r="A26" s="497" t="n">
+        <v>11</v>
+      </c>
+      <c r="B26" s="481" t="n"/>
+      <c r="C26" s="482" t="n"/>
+      <c r="D26" s="498" t="n"/>
+      <c r="E26" s="481" t="n"/>
+      <c r="F26" s="481" t="n"/>
+      <c r="G26" s="482" t="n"/>
+      <c r="H26" s="498" t="n"/>
+      <c r="I26" s="481" t="n"/>
+      <c r="J26" s="481" t="n"/>
+      <c r="K26" s="481" t="n"/>
+      <c r="L26" s="481" t="n"/>
+      <c r="M26" s="481" t="n"/>
+      <c r="N26" s="481" t="n"/>
+      <c r="O26" s="481" t="n"/>
+      <c r="P26" s="481" t="n"/>
+      <c r="Q26" s="481" t="n"/>
+      <c r="R26" s="481" t="n"/>
+      <c r="S26" s="481" t="n"/>
+      <c r="T26" s="482" t="n"/>
+      <c r="U26" s="498" t="n"/>
+      <c r="V26" s="481" t="n"/>
+      <c r="W26" s="481" t="n"/>
+      <c r="X26" s="481" t="n"/>
+      <c r="Y26" s="481" t="n"/>
+      <c r="Z26" s="481" t="n"/>
+      <c r="AA26" s="481" t="n"/>
+      <c r="AB26" s="481" t="n"/>
+      <c r="AC26" s="481" t="n"/>
+      <c r="AD26" s="482" t="n"/>
+      <c r="AE26" s="498" t="n"/>
+      <c r="AF26" s="481" t="n"/>
+      <c r="AG26" s="481" t="n"/>
+      <c r="AH26" s="481" t="n"/>
+      <c r="AI26" s="482" t="n"/>
+      <c r="AJ26" s="498" t="n"/>
+      <c r="AK26" s="481" t="n"/>
+      <c r="AL26" s="481" t="n"/>
+      <c r="AM26" s="481" t="n"/>
+      <c r="AN26" s="481" t="n"/>
+      <c r="AO26" s="481" t="n"/>
+      <c r="AP26" s="481" t="n"/>
+      <c r="AQ26" s="481" t="n"/>
+      <c r="AR26" s="482" t="n"/>
+      <c r="AS26" s="498" t="n"/>
+      <c r="AT26" s="481" t="n"/>
+      <c r="AU26" s="481" t="n"/>
+      <c r="AV26" s="481" t="n"/>
+      <c r="AW26" s="481" t="n"/>
+      <c r="AX26" s="482" t="n"/>
+      <c r="AY26" s="499" t="n"/>
+      <c r="AZ26" s="481" t="n"/>
+      <c r="BA26" s="481" t="n"/>
+      <c r="BB26" s="481" t="n"/>
+      <c r="BC26" s="481" t="n"/>
+      <c r="BD26" s="486" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" s="264">
+      <c r="A27" s="497" t="n">
+        <v>12</v>
+      </c>
+      <c r="B27" s="481" t="n"/>
+      <c r="C27" s="482" t="n"/>
+      <c r="D27" s="500" t="n"/>
+      <c r="E27" s="481" t="n"/>
+      <c r="F27" s="481" t="n"/>
+      <c r="G27" s="482" t="n"/>
+      <c r="H27" s="500" t="n"/>
+      <c r="I27" s="481" t="n"/>
+      <c r="J27" s="481" t="n"/>
+      <c r="K27" s="481" t="n"/>
+      <c r="L27" s="481" t="n"/>
+      <c r="M27" s="481" t="n"/>
+      <c r="N27" s="481" t="n"/>
+      <c r="O27" s="481" t="n"/>
+      <c r="P27" s="481" t="n"/>
+      <c r="Q27" s="481" t="n"/>
+      <c r="R27" s="481" t="n"/>
+      <c r="S27" s="481" t="n"/>
+      <c r="T27" s="482" t="n"/>
+      <c r="U27" s="500" t="n"/>
+      <c r="V27" s="481" t="n"/>
+      <c r="W27" s="481" t="n"/>
+      <c r="X27" s="481" t="n"/>
+      <c r="Y27" s="481" t="n"/>
+      <c r="Z27" s="481" t="n"/>
+      <c r="AA27" s="481" t="n"/>
+      <c r="AB27" s="481" t="n"/>
+      <c r="AC27" s="481" t="n"/>
+      <c r="AD27" s="482" t="n"/>
+      <c r="AE27" s="500" t="n"/>
+      <c r="AF27" s="481" t="n"/>
+      <c r="AG27" s="481" t="n"/>
+      <c r="AH27" s="481" t="n"/>
+      <c r="AI27" s="482" t="n"/>
+      <c r="AJ27" s="500" t="n"/>
+      <c r="AK27" s="481" t="n"/>
+      <c r="AL27" s="481" t="n"/>
+      <c r="AM27" s="481" t="n"/>
+      <c r="AN27" s="481" t="n"/>
+      <c r="AO27" s="481" t="n"/>
+      <c r="AP27" s="481" t="n"/>
+      <c r="AQ27" s="481" t="n"/>
+      <c r="AR27" s="482" t="n"/>
+      <c r="AS27" s="500" t="n"/>
+      <c r="AT27" s="481" t="n"/>
+      <c r="AU27" s="481" t="n"/>
+      <c r="AV27" s="481" t="n"/>
+      <c r="AW27" s="481" t="n"/>
+      <c r="AX27" s="482" t="n"/>
+      <c r="AY27" s="501" t="n"/>
+      <c r="AZ27" s="481" t="n"/>
+      <c r="BA27" s="481" t="n"/>
+      <c r="BB27" s="481" t="n"/>
+      <c r="BC27" s="481" t="n"/>
+      <c r="BD27" s="486" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" s="264">
+      <c r="A28" s="497" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" s="481" t="n"/>
+      <c r="C28" s="482" t="n"/>
+      <c r="D28" s="498" t="n"/>
+      <c r="E28" s="481" t="n"/>
+      <c r="F28" s="481" t="n"/>
+      <c r="G28" s="482" t="n"/>
+      <c r="H28" s="498" t="n"/>
+      <c r="I28" s="481" t="n"/>
+      <c r="J28" s="481" t="n"/>
+      <c r="K28" s="481" t="n"/>
+      <c r="L28" s="481" t="n"/>
+      <c r="M28" s="481" t="n"/>
+      <c r="N28" s="481" t="n"/>
+      <c r="O28" s="481" t="n"/>
+      <c r="P28" s="481" t="n"/>
+      <c r="Q28" s="481" t="n"/>
+      <c r="R28" s="481" t="n"/>
+      <c r="S28" s="481" t="n"/>
+      <c r="T28" s="482" t="n"/>
+      <c r="U28" s="498" t="n"/>
+      <c r="V28" s="481" t="n"/>
+      <c r="W28" s="481" t="n"/>
+      <c r="X28" s="481" t="n"/>
+      <c r="Y28" s="481" t="n"/>
+      <c r="Z28" s="481" t="n"/>
+      <c r="AA28" s="481" t="n"/>
+      <c r="AB28" s="481" t="n"/>
+      <c r="AC28" s="481" t="n"/>
+      <c r="AD28" s="482" t="n"/>
+      <c r="AE28" s="498" t="n"/>
+      <c r="AF28" s="481" t="n"/>
+      <c r="AG28" s="481" t="n"/>
+      <c r="AH28" s="481" t="n"/>
+      <c r="AI28" s="482" t="n"/>
+      <c r="AJ28" s="498" t="n"/>
+      <c r="AK28" s="481" t="n"/>
+      <c r="AL28" s="481" t="n"/>
+      <c r="AM28" s="481" t="n"/>
+      <c r="AN28" s="481" t="n"/>
+      <c r="AO28" s="481" t="n"/>
+      <c r="AP28" s="481" t="n"/>
+      <c r="AQ28" s="481" t="n"/>
+      <c r="AR28" s="482" t="n"/>
+      <c r="AS28" s="498" t="n"/>
+      <c r="AT28" s="481" t="n"/>
+      <c r="AU28" s="481" t="n"/>
+      <c r="AV28" s="481" t="n"/>
+      <c r="AW28" s="481" t="n"/>
+      <c r="AX28" s="482" t="n"/>
+      <c r="AY28" s="499" t="n"/>
+      <c r="AZ28" s="481" t="n"/>
+      <c r="BA28" s="481" t="n"/>
+      <c r="BB28" s="481" t="n"/>
+      <c r="BC28" s="481" t="n"/>
+      <c r="BD28" s="486" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" s="264">
+      <c r="A29" s="497" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" s="481" t="n"/>
+      <c r="C29" s="482" t="n"/>
+      <c r="D29" s="500" t="n"/>
+      <c r="E29" s="481" t="n"/>
+      <c r="F29" s="481" t="n"/>
+      <c r="G29" s="482" t="n"/>
+      <c r="H29" s="500" t="n"/>
+      <c r="I29" s="481" t="n"/>
+      <c r="J29" s="481" t="n"/>
+      <c r="K29" s="481" t="n"/>
+      <c r="L29" s="481" t="n"/>
+      <c r="M29" s="481" t="n"/>
+      <c r="N29" s="481" t="n"/>
+      <c r="O29" s="481" t="n"/>
+      <c r="P29" s="481" t="n"/>
+      <c r="Q29" s="481" t="n"/>
+      <c r="R29" s="481" t="n"/>
+      <c r="S29" s="481" t="n"/>
+      <c r="T29" s="482" t="n"/>
+      <c r="U29" s="500" t="n"/>
+      <c r="V29" s="481" t="n"/>
+      <c r="W29" s="481" t="n"/>
+      <c r="X29" s="481" t="n"/>
+      <c r="Y29" s="481" t="n"/>
+      <c r="Z29" s="481" t="n"/>
+      <c r="AA29" s="481" t="n"/>
+      <c r="AB29" s="481" t="n"/>
+      <c r="AC29" s="481" t="n"/>
+      <c r="AD29" s="482" t="n"/>
+      <c r="AE29" s="500" t="n"/>
+      <c r="AF29" s="481" t="n"/>
+      <c r="AG29" s="481" t="n"/>
+      <c r="AH29" s="481" t="n"/>
+      <c r="AI29" s="482" t="n"/>
+      <c r="AJ29" s="500" t="n"/>
+      <c r="AK29" s="481" t="n"/>
+      <c r="AL29" s="481" t="n"/>
+      <c r="AM29" s="481" t="n"/>
+      <c r="AN29" s="481" t="n"/>
+      <c r="AO29" s="481" t="n"/>
+      <c r="AP29" s="481" t="n"/>
+      <c r="AQ29" s="481" t="n"/>
+      <c r="AR29" s="482" t="n"/>
+      <c r="AS29" s="500" t="n"/>
+      <c r="AT29" s="481" t="n"/>
+      <c r="AU29" s="481" t="n"/>
+      <c r="AV29" s="481" t="n"/>
+      <c r="AW29" s="481" t="n"/>
+      <c r="AX29" s="482" t="n"/>
+      <c r="AY29" s="501" t="n"/>
+      <c r="AZ29" s="481" t="n"/>
+      <c r="BA29" s="481" t="n"/>
+      <c r="BB29" s="481" t="n"/>
+      <c r="BC29" s="481" t="n"/>
+      <c r="BD29" s="486" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" s="264">
+      <c r="A30" s="497" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" s="481" t="n"/>
+      <c r="C30" s="482" t="n"/>
+      <c r="D30" s="498" t="n"/>
+      <c r="E30" s="481" t="n"/>
+      <c r="F30" s="481" t="n"/>
+      <c r="G30" s="482" t="n"/>
+      <c r="H30" s="498" t="n"/>
+      <c r="I30" s="481" t="n"/>
+      <c r="J30" s="481" t="n"/>
+      <c r="K30" s="481" t="n"/>
+      <c r="L30" s="481" t="n"/>
+      <c r="M30" s="481" t="n"/>
+      <c r="N30" s="481" t="n"/>
+      <c r="O30" s="481" t="n"/>
+      <c r="P30" s="481" t="n"/>
+      <c r="Q30" s="481" t="n"/>
+      <c r="R30" s="481" t="n"/>
+      <c r="S30" s="481" t="n"/>
+      <c r="T30" s="482" t="n"/>
+      <c r="U30" s="498" t="n"/>
+      <c r="V30" s="481" t="n"/>
+      <c r="W30" s="481" t="n"/>
+      <c r="X30" s="481" t="n"/>
+      <c r="Y30" s="481" t="n"/>
+      <c r="Z30" s="481" t="n"/>
+      <c r="AA30" s="481" t="n"/>
+      <c r="AB30" s="481" t="n"/>
+      <c r="AC30" s="481" t="n"/>
+      <c r="AD30" s="482" t="n"/>
+      <c r="AE30" s="498" t="n"/>
+      <c r="AF30" s="481" t="n"/>
+      <c r="AG30" s="481" t="n"/>
+      <c r="AH30" s="481" t="n"/>
+      <c r="AI30" s="482" t="n"/>
+      <c r="AJ30" s="498" t="n"/>
+      <c r="AK30" s="481" t="n"/>
+      <c r="AL30" s="481" t="n"/>
+      <c r="AM30" s="481" t="n"/>
+      <c r="AN30" s="481" t="n"/>
+      <c r="AO30" s="481" t="n"/>
+      <c r="AP30" s="481" t="n"/>
+      <c r="AQ30" s="481" t="n"/>
+      <c r="AR30" s="482" t="n"/>
+      <c r="AS30" s="498" t="n"/>
+      <c r="AT30" s="481" t="n"/>
+      <c r="AU30" s="481" t="n"/>
+      <c r="AV30" s="481" t="n"/>
+      <c r="AW30" s="481" t="n"/>
+      <c r="AX30" s="482" t="n"/>
+      <c r="AY30" s="499" t="n"/>
+      <c r="AZ30" s="481" t="n"/>
+      <c r="BA30" s="481" t="n"/>
+      <c r="BB30" s="481" t="n"/>
+      <c r="BC30" s="481" t="n"/>
+      <c r="BD30" s="486" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" s="264">
+      <c r="A31" s="502" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="488" t="n"/>
-      <c r="C25" s="488" t="n"/>
-      <c r="D25" s="489" t="n"/>
-      <c r="E25" s="490" t="n"/>
-      <c r="F25" s="488" t="n"/>
-      <c r="G25" s="488" t="n"/>
-      <c r="H25" s="488" t="n"/>
-      <c r="I25" s="489" t="n"/>
-      <c r="J25" s="490" t="n"/>
-      <c r="K25" s="488" t="n"/>
-      <c r="L25" s="488" t="n"/>
-      <c r="M25" s="488" t="n"/>
-      <c r="N25" s="488" t="n"/>
-      <c r="O25" s="488" t="n"/>
-      <c r="P25" s="488" t="n"/>
-      <c r="Q25" s="488" t="n"/>
-      <c r="R25" s="488" t="n"/>
-      <c r="S25" s="488" t="n"/>
-      <c r="T25" s="488" t="n"/>
-      <c r="U25" s="488" t="n"/>
-      <c r="V25" s="489" t="n"/>
-      <c r="W25" s="490" t="n"/>
-      <c r="X25" s="488" t="n"/>
-      <c r="Y25" s="488" t="n"/>
-      <c r="Z25" s="488" t="n"/>
-      <c r="AA25" s="488" t="n"/>
-      <c r="AB25" s="488" t="n"/>
-      <c r="AC25" s="488" t="n"/>
-      <c r="AD25" s="488" t="n"/>
-      <c r="AE25" s="488" t="n"/>
-      <c r="AF25" s="488" t="n"/>
-      <c r="AG25" s="489" t="n"/>
-      <c r="AH25" s="490" t="n"/>
-      <c r="AI25" s="488" t="n"/>
-      <c r="AJ25" s="488" t="n"/>
-      <c r="AK25" s="488" t="n"/>
-      <c r="AL25" s="489" t="n"/>
-      <c r="AM25" s="490" t="n"/>
-      <c r="AN25" s="488" t="n"/>
-      <c r="AO25" s="488" t="n"/>
-      <c r="AP25" s="488" t="n"/>
-      <c r="AQ25" s="488" t="n"/>
-      <c r="AR25" s="488" t="n"/>
-      <c r="AS25" s="488" t="n"/>
-      <c r="AT25" s="488" t="n"/>
-      <c r="AU25" s="489" t="n"/>
-      <c r="AV25" s="490" t="n"/>
-      <c r="AW25" s="488" t="n"/>
-      <c r="AX25" s="488" t="n"/>
-      <c r="AY25" s="488" t="n"/>
-      <c r="AZ25" s="489" t="n"/>
-      <c r="BA25" s="491" t="n"/>
-      <c r="BB25" s="488" t="n"/>
-      <c r="BC25" s="488" t="n"/>
-      <c r="BD25" s="492" t="n"/>
+      <c r="B31" s="488" t="n"/>
+      <c r="C31" s="489" t="n"/>
+      <c r="D31" s="503" t="n"/>
+      <c r="E31" s="488" t="n"/>
+      <c r="F31" s="488" t="n"/>
+      <c r="G31" s="489" t="n"/>
+      <c r="H31" s="503" t="n"/>
+      <c r="I31" s="488" t="n"/>
+      <c r="J31" s="488" t="n"/>
+      <c r="K31" s="488" t="n"/>
+      <c r="L31" s="488" t="n"/>
+      <c r="M31" s="488" t="n"/>
+      <c r="N31" s="488" t="n"/>
+      <c r="O31" s="488" t="n"/>
+      <c r="P31" s="488" t="n"/>
+      <c r="Q31" s="488" t="n"/>
+      <c r="R31" s="488" t="n"/>
+      <c r="S31" s="488" t="n"/>
+      <c r="T31" s="489" t="n"/>
+      <c r="U31" s="503" t="n"/>
+      <c r="V31" s="488" t="n"/>
+      <c r="W31" s="488" t="n"/>
+      <c r="X31" s="488" t="n"/>
+      <c r="Y31" s="488" t="n"/>
+      <c r="Z31" s="488" t="n"/>
+      <c r="AA31" s="488" t="n"/>
+      <c r="AB31" s="488" t="n"/>
+      <c r="AC31" s="488" t="n"/>
+      <c r="AD31" s="489" t="n"/>
+      <c r="AE31" s="503" t="n"/>
+      <c r="AF31" s="488" t="n"/>
+      <c r="AG31" s="488" t="n"/>
+      <c r="AH31" s="488" t="n"/>
+      <c r="AI31" s="489" t="n"/>
+      <c r="AJ31" s="503" t="n"/>
+      <c r="AK31" s="488" t="n"/>
+      <c r="AL31" s="488" t="n"/>
+      <c r="AM31" s="488" t="n"/>
+      <c r="AN31" s="488" t="n"/>
+      <c r="AO31" s="488" t="n"/>
+      <c r="AP31" s="488" t="n"/>
+      <c r="AQ31" s="488" t="n"/>
+      <c r="AR31" s="489" t="n"/>
+      <c r="AS31" s="503" t="n"/>
+      <c r="AT31" s="488" t="n"/>
+      <c r="AU31" s="488" t="n"/>
+      <c r="AV31" s="488" t="n"/>
+      <c r="AW31" s="488" t="n"/>
+      <c r="AX31" s="489" t="n"/>
+      <c r="AY31" s="504" t="n"/>
+      <c r="AZ31" s="488" t="n"/>
+      <c r="BA31" s="488" t="n"/>
+      <c r="BB31" s="488" t="n"/>
+      <c r="BC31" s="488" t="n"/>
+      <c r="BD31" s="493" t="n"/>
     </row>
-    <row r="26" ht="4" customHeight="1" s="264">
-      <c r="A26" s="494" t="n"/>
-      <c r="B26" s="26" t="n"/>
-      <c r="C26" s="26" t="n"/>
-      <c r="D26" s="26" t="n"/>
-      <c r="E26" s="26" t="n"/>
-      <c r="F26" s="26" t="n"/>
-      <c r="G26" s="26" t="n"/>
-      <c r="H26" s="26" t="n"/>
-      <c r="I26" s="26" t="n"/>
-      <c r="J26" s="26" t="n"/>
-      <c r="K26" s="26" t="n"/>
-      <c r="L26" s="26" t="n"/>
-      <c r="M26" s="26" t="n"/>
-      <c r="N26" s="26" t="n"/>
-      <c r="O26" s="26" t="n"/>
-      <c r="P26" s="26" t="n"/>
-      <c r="Q26" s="26" t="n"/>
-      <c r="R26" s="26" t="n"/>
-      <c r="S26" s="26" t="n"/>
-      <c r="T26" s="26" t="n"/>
-      <c r="U26" s="26" t="n"/>
-      <c r="V26" s="26" t="n"/>
-      <c r="W26" s="26" t="n"/>
-      <c r="X26" s="26" t="n"/>
-      <c r="Y26" s="26" t="n"/>
-      <c r="Z26" s="26" t="n"/>
-      <c r="AA26" s="26" t="n"/>
-      <c r="AB26" s="26" t="n"/>
-      <c r="AC26" s="26" t="n"/>
-      <c r="AD26" s="26" t="n"/>
-      <c r="AE26" s="26" t="n"/>
-      <c r="AF26" s="26" t="n"/>
-      <c r="AG26" s="26" t="n"/>
-      <c r="AH26" s="26" t="n"/>
-      <c r="AI26" s="26" t="n"/>
-      <c r="AJ26" s="26" t="n"/>
-      <c r="AK26" s="26" t="n"/>
-      <c r="AL26" s="26" t="n"/>
-      <c r="AM26" s="26" t="n"/>
-      <c r="AN26" s="26" t="n"/>
-      <c r="AO26" s="26" t="n"/>
-      <c r="AP26" s="26" t="n"/>
-      <c r="AQ26" s="26" t="n"/>
-      <c r="AR26" s="26" t="n"/>
-      <c r="AS26" s="26" t="n"/>
-      <c r="AT26" s="26" t="n"/>
-      <c r="AU26" s="26" t="n"/>
-      <c r="AV26" s="26" t="n"/>
-      <c r="AW26" s="26" t="n"/>
-      <c r="AX26" s="26" t="n"/>
-      <c r="AY26" s="26" t="n"/>
-      <c r="AZ26" s="26" t="n"/>
-      <c r="BA26" s="26" t="n"/>
-      <c r="BB26" s="26" t="n"/>
-      <c r="BC26" s="26" t="n"/>
-      <c r="BD26" s="26" t="n"/>
+    <row r="32" ht="4" customHeight="1" s="264">
+      <c r="A32" s="469" t="n"/>
+      <c r="B32" s="26" t="n"/>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="26" t="n"/>
+      <c r="E32" s="26" t="n"/>
+      <c r="F32" s="26" t="n"/>
+      <c r="G32" s="26" t="n"/>
+      <c r="H32" s="26" t="n"/>
+      <c r="I32" s="26" t="n"/>
+      <c r="J32" s="26" t="n"/>
+      <c r="K32" s="26" t="n"/>
+      <c r="L32" s="26" t="n"/>
+      <c r="M32" s="26" t="n"/>
+      <c r="N32" s="26" t="n"/>
+      <c r="O32" s="26" t="n"/>
+      <c r="P32" s="26" t="n"/>
+      <c r="Q32" s="26" t="n"/>
+      <c r="R32" s="26" t="n"/>
+      <c r="S32" s="26" t="n"/>
+      <c r="T32" s="26" t="n"/>
+      <c r="U32" s="26" t="n"/>
+      <c r="V32" s="26" t="n"/>
+      <c r="W32" s="26" t="n"/>
+      <c r="X32" s="26" t="n"/>
+      <c r="Y32" s="26" t="n"/>
+      <c r="Z32" s="26" t="n"/>
+      <c r="AA32" s="26" t="n"/>
+      <c r="AB32" s="26" t="n"/>
+      <c r="AC32" s="26" t="n"/>
+      <c r="AD32" s="26" t="n"/>
+      <c r="AE32" s="26" t="n"/>
+      <c r="AF32" s="26" t="n"/>
+      <c r="AG32" s="26" t="n"/>
+      <c r="AH32" s="26" t="n"/>
+      <c r="AI32" s="26" t="n"/>
+      <c r="AJ32" s="26" t="n"/>
+      <c r="AK32" s="26" t="n"/>
+      <c r="AL32" s="26" t="n"/>
+      <c r="AM32" s="26" t="n"/>
+      <c r="AN32" s="26" t="n"/>
+      <c r="AO32" s="26" t="n"/>
+      <c r="AP32" s="26" t="n"/>
+      <c r="AQ32" s="26" t="n"/>
+      <c r="AR32" s="26" t="n"/>
+      <c r="AS32" s="26" t="n"/>
+      <c r="AT32" s="26" t="n"/>
+      <c r="AU32" s="26" t="n"/>
+      <c r="AV32" s="26" t="n"/>
+      <c r="AW32" s="26" t="n"/>
+      <c r="AX32" s="26" t="n"/>
+      <c r="AY32" s="26" t="n"/>
+      <c r="AZ32" s="26" t="n"/>
+      <c r="BA32" s="26" t="n"/>
+      <c r="BB32" s="26" t="n"/>
+      <c r="BC32" s="26" t="n"/>
+      <c r="BD32" s="26" t="n"/>
     </row>
-    <row r="27" ht="24" customHeight="1" s="264">
-      <c r="A27" s="493" t="inlineStr">
-        <is>
-          <t>NOTICE — Every dimension, note and GD&amp;T callout on the drawing must carry a unique balloon and a row here. This sheet is the master index for FAI (FRM-311) and in-process inspection (FRM-622). Ref: SOP-301. Retain: life of part.</t>
-        </is>
-      </c>
-      <c r="B27" s="471" t="n"/>
-      <c r="C27" s="471" t="n"/>
-      <c r="D27" s="471" t="n"/>
-      <c r="E27" s="471" t="n"/>
-      <c r="F27" s="471" t="n"/>
-      <c r="G27" s="471" t="n"/>
-      <c r="H27" s="471" t="n"/>
-      <c r="I27" s="471" t="n"/>
-      <c r="J27" s="471" t="n"/>
-      <c r="K27" s="471" t="n"/>
-      <c r="L27" s="471" t="n"/>
-      <c r="M27" s="471" t="n"/>
-      <c r="N27" s="471" t="n"/>
-      <c r="O27" s="471" t="n"/>
-      <c r="P27" s="471" t="n"/>
-      <c r="Q27" s="471" t="n"/>
-      <c r="R27" s="471" t="n"/>
-      <c r="S27" s="471" t="n"/>
-      <c r="T27" s="471" t="n"/>
-      <c r="U27" s="471" t="n"/>
-      <c r="V27" s="471" t="n"/>
-      <c r="W27" s="471" t="n"/>
-      <c r="X27" s="471" t="n"/>
-      <c r="Y27" s="471" t="n"/>
-      <c r="Z27" s="471" t="n"/>
-      <c r="AA27" s="471" t="n"/>
-      <c r="AB27" s="471" t="n"/>
-      <c r="AC27" s="471" t="n"/>
-      <c r="AD27" s="471" t="n"/>
-      <c r="AE27" s="471" t="n"/>
-      <c r="AF27" s="471" t="n"/>
-      <c r="AG27" s="471" t="n"/>
-      <c r="AH27" s="471" t="n"/>
-      <c r="AI27" s="471" t="n"/>
-      <c r="AJ27" s="471" t="n"/>
-      <c r="AK27" s="471" t="n"/>
-      <c r="AL27" s="471" t="n"/>
-      <c r="AM27" s="471" t="n"/>
-      <c r="AN27" s="471" t="n"/>
-      <c r="AO27" s="471" t="n"/>
-      <c r="AP27" s="471" t="n"/>
-      <c r="AQ27" s="471" t="n"/>
-      <c r="AR27" s="471" t="n"/>
-      <c r="AS27" s="471" t="n"/>
-      <c r="AT27" s="471" t="n"/>
-      <c r="AU27" s="471" t="n"/>
-      <c r="AV27" s="471" t="n"/>
-      <c r="AW27" s="471" t="n"/>
-      <c r="AX27" s="471" t="n"/>
-      <c r="AY27" s="471" t="n"/>
-      <c r="AZ27" s="471" t="n"/>
-      <c r="BA27" s="471" t="n"/>
-      <c r="BB27" s="471" t="n"/>
-      <c r="BC27" s="471" t="n"/>
-      <c r="BD27" s="472" t="n"/>
+    <row r="33" ht="17" customHeight="1" s="264">
+      <c r="A33" s="470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3.  ACCOUNTABILITY REVIEW</t>
+        </is>
+      </c>
+      <c r="B33" s="471" t="n"/>
+      <c r="C33" s="471" t="n"/>
+      <c r="D33" s="471" t="n"/>
+      <c r="E33" s="471" t="n"/>
+      <c r="F33" s="471" t="n"/>
+      <c r="G33" s="471" t="n"/>
+      <c r="H33" s="471" t="n"/>
+      <c r="I33" s="471" t="n"/>
+      <c r="J33" s="471" t="n"/>
+      <c r="K33" s="471" t="n"/>
+      <c r="L33" s="471" t="n"/>
+      <c r="M33" s="471" t="n"/>
+      <c r="N33" s="471" t="n"/>
+      <c r="O33" s="471" t="n"/>
+      <c r="P33" s="471" t="n"/>
+      <c r="Q33" s="471" t="n"/>
+      <c r="R33" s="471" t="n"/>
+      <c r="S33" s="471" t="n"/>
+      <c r="T33" s="471" t="n"/>
+      <c r="U33" s="471" t="n"/>
+      <c r="V33" s="471" t="n"/>
+      <c r="W33" s="471" t="n"/>
+      <c r="X33" s="471" t="n"/>
+      <c r="Y33" s="471" t="n"/>
+      <c r="Z33" s="471" t="n"/>
+      <c r="AA33" s="471" t="n"/>
+      <c r="AB33" s="471" t="n"/>
+      <c r="AC33" s="471" t="n"/>
+      <c r="AD33" s="471" t="n"/>
+      <c r="AE33" s="471" t="n"/>
+      <c r="AF33" s="471" t="n"/>
+      <c r="AG33" s="471" t="n"/>
+      <c r="AH33" s="471" t="n"/>
+      <c r="AI33" s="471" t="n"/>
+      <c r="AJ33" s="471" t="n"/>
+      <c r="AK33" s="471" t="n"/>
+      <c r="AL33" s="471" t="n"/>
+      <c r="AM33" s="471" t="n"/>
+      <c r="AN33" s="471" t="n"/>
+      <c r="AO33" s="471" t="n"/>
+      <c r="AP33" s="471" t="n"/>
+      <c r="AQ33" s="471" t="n"/>
+      <c r="AR33" s="471" t="n"/>
+      <c r="AS33" s="471" t="n"/>
+      <c r="AT33" s="471" t="n"/>
+      <c r="AU33" s="471" t="n"/>
+      <c r="AV33" s="471" t="n"/>
+      <c r="AW33" s="471" t="n"/>
+      <c r="AX33" s="471" t="n"/>
+      <c r="AY33" s="471" t="n"/>
+      <c r="AZ33" s="471" t="n"/>
+      <c r="BA33" s="471" t="n"/>
+      <c r="BB33" s="471" t="n"/>
+      <c r="BC33" s="471" t="n"/>
+      <c r="BD33" s="472" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" s="264">
+      <c r="A34" s="473" t="inlineStr">
+        <is>
+          <t>CTQ Count</t>
+        </is>
+      </c>
+      <c r="B34" s="474" t="n"/>
+      <c r="C34" s="474" t="n"/>
+      <c r="D34" s="474" t="n"/>
+      <c r="E34" s="474" t="n"/>
+      <c r="F34" s="474" t="n"/>
+      <c r="G34" s="474" t="n"/>
+      <c r="H34" s="474" t="n"/>
+      <c r="I34" s="474" t="n"/>
+      <c r="J34" s="475" t="n"/>
+      <c r="K34" s="476" t="n"/>
+      <c r="L34" s="474" t="n"/>
+      <c r="M34" s="474" t="n"/>
+      <c r="N34" s="474" t="n"/>
+      <c r="O34" s="474" t="n"/>
+      <c r="P34" s="474" t="n"/>
+      <c r="Q34" s="474" t="n"/>
+      <c r="R34" s="474" t="n"/>
+      <c r="S34" s="474" t="n"/>
+      <c r="T34" s="474" t="n"/>
+      <c r="U34" s="474" t="n"/>
+      <c r="V34" s="474" t="n"/>
+      <c r="W34" s="474" t="n"/>
+      <c r="X34" s="474" t="n"/>
+      <c r="Y34" s="474" t="n"/>
+      <c r="Z34" s="474" t="n"/>
+      <c r="AA34" s="474" t="n"/>
+      <c r="AB34" s="475" t="n"/>
+      <c r="AC34" s="477" t="inlineStr">
+        <is>
+          <t>KPC Count</t>
+        </is>
+      </c>
+      <c r="AD34" s="474" t="n"/>
+      <c r="AE34" s="474" t="n"/>
+      <c r="AF34" s="474" t="n"/>
+      <c r="AG34" s="474" t="n"/>
+      <c r="AH34" s="474" t="n"/>
+      <c r="AI34" s="474" t="n"/>
+      <c r="AJ34" s="474" t="n"/>
+      <c r="AK34" s="474" t="n"/>
+      <c r="AL34" s="475" t="n"/>
+      <c r="AM34" s="478" t="n"/>
+      <c r="AN34" s="474" t="n"/>
+      <c r="AO34" s="474" t="n"/>
+      <c r="AP34" s="474" t="n"/>
+      <c r="AQ34" s="474" t="n"/>
+      <c r="AR34" s="474" t="n"/>
+      <c r="AS34" s="474" t="n"/>
+      <c r="AT34" s="474" t="n"/>
+      <c r="AU34" s="474" t="n"/>
+      <c r="AV34" s="474" t="n"/>
+      <c r="AW34" s="474" t="n"/>
+      <c r="AX34" s="474" t="n"/>
+      <c r="AY34" s="474" t="n"/>
+      <c r="AZ34" s="474" t="n"/>
+      <c r="BA34" s="474" t="n"/>
+      <c r="BB34" s="474" t="n"/>
+      <c r="BC34" s="474" t="n"/>
+      <c r="BD34" s="479" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" s="264">
+      <c r="A35" s="480" t="inlineStr">
+        <is>
+          <t>All Characteristics Ballooned? (Yes / No)</t>
+        </is>
+      </c>
+      <c r="B35" s="481" t="n"/>
+      <c r="C35" s="481" t="n"/>
+      <c r="D35" s="481" t="n"/>
+      <c r="E35" s="481" t="n"/>
+      <c r="F35" s="481" t="n"/>
+      <c r="G35" s="481" t="n"/>
+      <c r="H35" s="481" t="n"/>
+      <c r="I35" s="481" t="n"/>
+      <c r="J35" s="482" t="n"/>
+      <c r="K35" s="483" t="n"/>
+      <c r="L35" s="481" t="n"/>
+      <c r="M35" s="481" t="n"/>
+      <c r="N35" s="481" t="n"/>
+      <c r="O35" s="481" t="n"/>
+      <c r="P35" s="481" t="n"/>
+      <c r="Q35" s="481" t="n"/>
+      <c r="R35" s="481" t="n"/>
+      <c r="S35" s="481" t="n"/>
+      <c r="T35" s="481" t="n"/>
+      <c r="U35" s="481" t="n"/>
+      <c r="V35" s="481" t="n"/>
+      <c r="W35" s="481" t="n"/>
+      <c r="X35" s="481" t="n"/>
+      <c r="Y35" s="481" t="n"/>
+      <c r="Z35" s="481" t="n"/>
+      <c r="AA35" s="481" t="n"/>
+      <c r="AB35" s="482" t="n"/>
+      <c r="AC35" s="484" t="inlineStr">
+        <is>
+          <t>Drawing Notes Captured? (Yes / No)</t>
+        </is>
+      </c>
+      <c r="AD35" s="481" t="n"/>
+      <c r="AE35" s="481" t="n"/>
+      <c r="AF35" s="481" t="n"/>
+      <c r="AG35" s="481" t="n"/>
+      <c r="AH35" s="481" t="n"/>
+      <c r="AI35" s="481" t="n"/>
+      <c r="AJ35" s="481" t="n"/>
+      <c r="AK35" s="481" t="n"/>
+      <c r="AL35" s="482" t="n"/>
+      <c r="AM35" s="485" t="n"/>
+      <c r="AN35" s="481" t="n"/>
+      <c r="AO35" s="481" t="n"/>
+      <c r="AP35" s="481" t="n"/>
+      <c r="AQ35" s="481" t="n"/>
+      <c r="AR35" s="481" t="n"/>
+      <c r="AS35" s="481" t="n"/>
+      <c r="AT35" s="481" t="n"/>
+      <c r="AU35" s="481" t="n"/>
+      <c r="AV35" s="481" t="n"/>
+      <c r="AW35" s="481" t="n"/>
+      <c r="AX35" s="481" t="n"/>
+      <c r="AY35" s="481" t="n"/>
+      <c r="AZ35" s="481" t="n"/>
+      <c r="BA35" s="481" t="n"/>
+      <c r="BB35" s="481" t="n"/>
+      <c r="BC35" s="481" t="n"/>
+      <c r="BD35" s="486" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" s="264">
+      <c r="A36" s="487" t="inlineStr">
+        <is>
+          <t>Engineering Review Note</t>
+        </is>
+      </c>
+      <c r="B36" s="488" t="n"/>
+      <c r="C36" s="488" t="n"/>
+      <c r="D36" s="488" t="n"/>
+      <c r="E36" s="488" t="n"/>
+      <c r="F36" s="488" t="n"/>
+      <c r="G36" s="488" t="n"/>
+      <c r="H36" s="488" t="n"/>
+      <c r="I36" s="488" t="n"/>
+      <c r="J36" s="489" t="n"/>
+      <c r="K36" s="490" t="n"/>
+      <c r="L36" s="488" t="n"/>
+      <c r="M36" s="488" t="n"/>
+      <c r="N36" s="488" t="n"/>
+      <c r="O36" s="488" t="n"/>
+      <c r="P36" s="488" t="n"/>
+      <c r="Q36" s="488" t="n"/>
+      <c r="R36" s="488" t="n"/>
+      <c r="S36" s="488" t="n"/>
+      <c r="T36" s="488" t="n"/>
+      <c r="U36" s="488" t="n"/>
+      <c r="V36" s="488" t="n"/>
+      <c r="W36" s="488" t="n"/>
+      <c r="X36" s="488" t="n"/>
+      <c r="Y36" s="488" t="n"/>
+      <c r="Z36" s="488" t="n"/>
+      <c r="AA36" s="488" t="n"/>
+      <c r="AB36" s="489" t="n"/>
+      <c r="AC36" s="491" t="inlineStr">
+        <is>
+          <t>QA Approval Ref</t>
+        </is>
+      </c>
+      <c r="AD36" s="488" t="n"/>
+      <c r="AE36" s="488" t="n"/>
+      <c r="AF36" s="488" t="n"/>
+      <c r="AG36" s="488" t="n"/>
+      <c r="AH36" s="488" t="n"/>
+      <c r="AI36" s="488" t="n"/>
+      <c r="AJ36" s="488" t="n"/>
+      <c r="AK36" s="488" t="n"/>
+      <c r="AL36" s="489" t="n"/>
+      <c r="AM36" s="492" t="n"/>
+      <c r="AN36" s="488" t="n"/>
+      <c r="AO36" s="488" t="n"/>
+      <c r="AP36" s="488" t="n"/>
+      <c r="AQ36" s="488" t="n"/>
+      <c r="AR36" s="488" t="n"/>
+      <c r="AS36" s="488" t="n"/>
+      <c r="AT36" s="488" t="n"/>
+      <c r="AU36" s="488" t="n"/>
+      <c r="AV36" s="488" t="n"/>
+      <c r="AW36" s="488" t="n"/>
+      <c r="AX36" s="488" t="n"/>
+      <c r="AY36" s="488" t="n"/>
+      <c r="AZ36" s="488" t="n"/>
+      <c r="BA36" s="488" t="n"/>
+      <c r="BB36" s="488" t="n"/>
+      <c r="BC36" s="488" t="n"/>
+      <c r="BD36" s="493" t="n"/>
+    </row>
+    <row r="37" ht="4" customHeight="1" s="264">
+      <c r="A37" s="469" t="n"/>
+      <c r="B37" s="26" t="n"/>
+      <c r="C37" s="26" t="n"/>
+      <c r="D37" s="26" t="n"/>
+      <c r="E37" s="26" t="n"/>
+      <c r="F37" s="26" t="n"/>
+      <c r="G37" s="26" t="n"/>
+      <c r="H37" s="26" t="n"/>
+      <c r="I37" s="26" t="n"/>
+      <c r="J37" s="26" t="n"/>
+      <c r="K37" s="26" t="n"/>
+      <c r="L37" s="26" t="n"/>
+      <c r="M37" s="26" t="n"/>
+      <c r="N37" s="26" t="n"/>
+      <c r="O37" s="26" t="n"/>
+      <c r="P37" s="26" t="n"/>
+      <c r="Q37" s="26" t="n"/>
+      <c r="R37" s="26" t="n"/>
+      <c r="S37" s="26" t="n"/>
+      <c r="T37" s="26" t="n"/>
+      <c r="U37" s="26" t="n"/>
+      <c r="V37" s="26" t="n"/>
+      <c r="W37" s="26" t="n"/>
+      <c r="X37" s="26" t="n"/>
+      <c r="Y37" s="26" t="n"/>
+      <c r="Z37" s="26" t="n"/>
+      <c r="AA37" s="26" t="n"/>
+      <c r="AB37" s="26" t="n"/>
+      <c r="AC37" s="26" t="n"/>
+      <c r="AD37" s="26" t="n"/>
+      <c r="AE37" s="26" t="n"/>
+      <c r="AF37" s="26" t="n"/>
+      <c r="AG37" s="26" t="n"/>
+      <c r="AH37" s="26" t="n"/>
+      <c r="AI37" s="26" t="n"/>
+      <c r="AJ37" s="26" t="n"/>
+      <c r="AK37" s="26" t="n"/>
+      <c r="AL37" s="26" t="n"/>
+      <c r="AM37" s="26" t="n"/>
+      <c r="AN37" s="26" t="n"/>
+      <c r="AO37" s="26" t="n"/>
+      <c r="AP37" s="26" t="n"/>
+      <c r="AQ37" s="26" t="n"/>
+      <c r="AR37" s="26" t="n"/>
+      <c r="AS37" s="26" t="n"/>
+      <c r="AT37" s="26" t="n"/>
+      <c r="AU37" s="26" t="n"/>
+      <c r="AV37" s="26" t="n"/>
+      <c r="AW37" s="26" t="n"/>
+      <c r="AX37" s="26" t="n"/>
+      <c r="AY37" s="26" t="n"/>
+      <c r="AZ37" s="26" t="n"/>
+      <c r="BA37" s="26" t="n"/>
+      <c r="BB37" s="26" t="n"/>
+      <c r="BC37" s="26" t="n"/>
+      <c r="BD37" s="26" t="n"/>
+    </row>
+    <row r="38" ht="17" customHeight="1" s="264">
+      <c r="A38" s="470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.  APPROVAL</t>
+        </is>
+      </c>
+      <c r="B38" s="471" t="n"/>
+      <c r="C38" s="471" t="n"/>
+      <c r="D38" s="471" t="n"/>
+      <c r="E38" s="471" t="n"/>
+      <c r="F38" s="471" t="n"/>
+      <c r="G38" s="471" t="n"/>
+      <c r="H38" s="471" t="n"/>
+      <c r="I38" s="471" t="n"/>
+      <c r="J38" s="471" t="n"/>
+      <c r="K38" s="471" t="n"/>
+      <c r="L38" s="471" t="n"/>
+      <c r="M38" s="471" t="n"/>
+      <c r="N38" s="471" t="n"/>
+      <c r="O38" s="471" t="n"/>
+      <c r="P38" s="471" t="n"/>
+      <c r="Q38" s="471" t="n"/>
+      <c r="R38" s="471" t="n"/>
+      <c r="S38" s="471" t="n"/>
+      <c r="T38" s="471" t="n"/>
+      <c r="U38" s="471" t="n"/>
+      <c r="V38" s="471" t="n"/>
+      <c r="W38" s="471" t="n"/>
+      <c r="X38" s="471" t="n"/>
+      <c r="Y38" s="471" t="n"/>
+      <c r="Z38" s="471" t="n"/>
+      <c r="AA38" s="471" t="n"/>
+      <c r="AB38" s="471" t="n"/>
+      <c r="AC38" s="471" t="n"/>
+      <c r="AD38" s="471" t="n"/>
+      <c r="AE38" s="471" t="n"/>
+      <c r="AF38" s="471" t="n"/>
+      <c r="AG38" s="471" t="n"/>
+      <c r="AH38" s="471" t="n"/>
+      <c r="AI38" s="471" t="n"/>
+      <c r="AJ38" s="471" t="n"/>
+      <c r="AK38" s="471" t="n"/>
+      <c r="AL38" s="471" t="n"/>
+      <c r="AM38" s="471" t="n"/>
+      <c r="AN38" s="471" t="n"/>
+      <c r="AO38" s="471" t="n"/>
+      <c r="AP38" s="471" t="n"/>
+      <c r="AQ38" s="471" t="n"/>
+      <c r="AR38" s="471" t="n"/>
+      <c r="AS38" s="471" t="n"/>
+      <c r="AT38" s="471" t="n"/>
+      <c r="AU38" s="471" t="n"/>
+      <c r="AV38" s="471" t="n"/>
+      <c r="AW38" s="471" t="n"/>
+      <c r="AX38" s="471" t="n"/>
+      <c r="AY38" s="471" t="n"/>
+      <c r="AZ38" s="471" t="n"/>
+      <c r="BA38" s="471" t="n"/>
+      <c r="BB38" s="471" t="n"/>
+      <c r="BC38" s="471" t="n"/>
+      <c r="BD38" s="472" t="n"/>
+    </row>
+    <row r="39" ht="17" customHeight="1" s="264">
+      <c r="A39" s="505" t="inlineStr">
+        <is>
+          <t>Quality Engineer</t>
+        </is>
+      </c>
+      <c r="B39" s="471" t="n"/>
+      <c r="C39" s="471" t="n"/>
+      <c r="D39" s="471" t="n"/>
+      <c r="E39" s="471" t="n"/>
+      <c r="F39" s="471" t="n"/>
+      <c r="G39" s="471" t="n"/>
+      <c r="H39" s="471" t="n"/>
+      <c r="I39" s="471" t="n"/>
+      <c r="J39" s="471" t="n"/>
+      <c r="K39" s="471" t="n"/>
+      <c r="L39" s="471" t="n"/>
+      <c r="M39" s="471" t="n"/>
+      <c r="N39" s="471" t="n"/>
+      <c r="O39" s="471" t="n"/>
+      <c r="P39" s="471" t="n"/>
+      <c r="Q39" s="471" t="n"/>
+      <c r="R39" s="472" t="n"/>
+      <c r="S39" s="505" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="T39" s="471" t="n"/>
+      <c r="U39" s="471" t="n"/>
+      <c r="V39" s="471" t="n"/>
+      <c r="W39" s="471" t="n"/>
+      <c r="X39" s="471" t="n"/>
+      <c r="Y39" s="471" t="n"/>
+      <c r="Z39" s="471" t="n"/>
+      <c r="AA39" s="471" t="n"/>
+      <c r="AB39" s="471" t="n"/>
+      <c r="AC39" s="471" t="n"/>
+      <c r="AD39" s="471" t="n"/>
+      <c r="AE39" s="471" t="n"/>
+      <c r="AF39" s="471" t="n"/>
+      <c r="AG39" s="471" t="n"/>
+      <c r="AH39" s="471" t="n"/>
+      <c r="AI39" s="471" t="n"/>
+      <c r="AJ39" s="471" t="n"/>
+      <c r="AK39" s="472" t="n"/>
+      <c r="AL39" s="505" t="inlineStr">
+        <is>
+          <t>QA Manager</t>
+        </is>
+      </c>
+      <c r="AM39" s="471" t="n"/>
+      <c r="AN39" s="471" t="n"/>
+      <c r="AO39" s="471" t="n"/>
+      <c r="AP39" s="471" t="n"/>
+      <c r="AQ39" s="471" t="n"/>
+      <c r="AR39" s="471" t="n"/>
+      <c r="AS39" s="471" t="n"/>
+      <c r="AT39" s="471" t="n"/>
+      <c r="AU39" s="471" t="n"/>
+      <c r="AV39" s="471" t="n"/>
+      <c r="AW39" s="471" t="n"/>
+      <c r="AX39" s="471" t="n"/>
+      <c r="AY39" s="471" t="n"/>
+      <c r="AZ39" s="471" t="n"/>
+      <c r="BA39" s="471" t="n"/>
+      <c r="BB39" s="471" t="n"/>
+      <c r="BC39" s="471" t="n"/>
+      <c r="BD39" s="472" t="n"/>
+    </row>
+    <row r="40" ht="26" customHeight="1" s="264">
+      <c r="A40" s="506" t="inlineStr">
+        <is>
+          <t>Name  /  Signature  /  Date</t>
+        </is>
+      </c>
+      <c r="B40" s="507" t="n"/>
+      <c r="C40" s="507" t="n"/>
+      <c r="D40" s="507" t="n"/>
+      <c r="E40" s="507" t="n"/>
+      <c r="F40" s="507" t="n"/>
+      <c r="G40" s="507" t="n"/>
+      <c r="H40" s="507" t="n"/>
+      <c r="I40" s="507" t="n"/>
+      <c r="J40" s="507" t="n"/>
+      <c r="K40" s="507" t="n"/>
+      <c r="L40" s="507" t="n"/>
+      <c r="M40" s="507" t="n"/>
+      <c r="N40" s="507" t="n"/>
+      <c r="O40" s="507" t="n"/>
+      <c r="P40" s="507" t="n"/>
+      <c r="Q40" s="507" t="n"/>
+      <c r="R40" s="508" t="n"/>
+      <c r="S40" s="506" t="inlineStr">
+        <is>
+          <t>Name  /  Signature  /  Date</t>
+        </is>
+      </c>
+      <c r="T40" s="507" t="n"/>
+      <c r="U40" s="507" t="n"/>
+      <c r="V40" s="507" t="n"/>
+      <c r="W40" s="507" t="n"/>
+      <c r="X40" s="507" t="n"/>
+      <c r="Y40" s="507" t="n"/>
+      <c r="Z40" s="507" t="n"/>
+      <c r="AA40" s="507" t="n"/>
+      <c r="AB40" s="507" t="n"/>
+      <c r="AC40" s="507" t="n"/>
+      <c r="AD40" s="507" t="n"/>
+      <c r="AE40" s="507" t="n"/>
+      <c r="AF40" s="507" t="n"/>
+      <c r="AG40" s="507" t="n"/>
+      <c r="AH40" s="507" t="n"/>
+      <c r="AI40" s="507" t="n"/>
+      <c r="AJ40" s="507" t="n"/>
+      <c r="AK40" s="508" t="n"/>
+      <c r="AL40" s="506" t="inlineStr">
+        <is>
+          <t>Name  /  Signature  /  Date</t>
+        </is>
+      </c>
+      <c r="AM40" s="507" t="n"/>
+      <c r="AN40" s="507" t="n"/>
+      <c r="AO40" s="507" t="n"/>
+      <c r="AP40" s="507" t="n"/>
+      <c r="AQ40" s="507" t="n"/>
+      <c r="AR40" s="507" t="n"/>
+      <c r="AS40" s="507" t="n"/>
+      <c r="AT40" s="507" t="n"/>
+      <c r="AU40" s="507" t="n"/>
+      <c r="AV40" s="507" t="n"/>
+      <c r="AW40" s="507" t="n"/>
+      <c r="AX40" s="507" t="n"/>
+      <c r="AY40" s="507" t="n"/>
+      <c r="AZ40" s="507" t="n"/>
+      <c r="BA40" s="507" t="n"/>
+      <c r="BB40" s="507" t="n"/>
+      <c r="BC40" s="507" t="n"/>
+      <c r="BD40" s="508" t="n"/>
+    </row>
+    <row r="41" ht="26" customHeight="1" s="264">
+      <c r="A41" s="509" t="n"/>
+      <c r="R41" s="510" t="n"/>
+      <c r="S41" s="509" t="n"/>
+      <c r="AK41" s="510" t="n"/>
+      <c r="AL41" s="509" t="n"/>
+      <c r="BD41" s="510" t="n"/>
+    </row>
+    <row r="42" ht="26" customHeight="1" s="264">
+      <c r="A42" s="511" t="n"/>
+      <c r="B42" s="488" t="n"/>
+      <c r="C42" s="488" t="n"/>
+      <c r="D42" s="488" t="n"/>
+      <c r="E42" s="488" t="n"/>
+      <c r="F42" s="488" t="n"/>
+      <c r="G42" s="488" t="n"/>
+      <c r="H42" s="488" t="n"/>
+      <c r="I42" s="488" t="n"/>
+      <c r="J42" s="488" t="n"/>
+      <c r="K42" s="488" t="n"/>
+      <c r="L42" s="488" t="n"/>
+      <c r="M42" s="488" t="n"/>
+      <c r="N42" s="488" t="n"/>
+      <c r="O42" s="488" t="n"/>
+      <c r="P42" s="488" t="n"/>
+      <c r="Q42" s="488" t="n"/>
+      <c r="R42" s="493" t="n"/>
+      <c r="S42" s="511" t="n"/>
+      <c r="T42" s="488" t="n"/>
+      <c r="U42" s="488" t="n"/>
+      <c r="V42" s="488" t="n"/>
+      <c r="W42" s="488" t="n"/>
+      <c r="X42" s="488" t="n"/>
+      <c r="Y42" s="488" t="n"/>
+      <c r="Z42" s="488" t="n"/>
+      <c r="AA42" s="488" t="n"/>
+      <c r="AB42" s="488" t="n"/>
+      <c r="AC42" s="488" t="n"/>
+      <c r="AD42" s="488" t="n"/>
+      <c r="AE42" s="488" t="n"/>
+      <c r="AF42" s="488" t="n"/>
+      <c r="AG42" s="488" t="n"/>
+      <c r="AH42" s="488" t="n"/>
+      <c r="AI42" s="488" t="n"/>
+      <c r="AJ42" s="488" t="n"/>
+      <c r="AK42" s="493" t="n"/>
+      <c r="AL42" s="511" t="n"/>
+      <c r="AM42" s="488" t="n"/>
+      <c r="AN42" s="488" t="n"/>
+      <c r="AO42" s="488" t="n"/>
+      <c r="AP42" s="488" t="n"/>
+      <c r="AQ42" s="488" t="n"/>
+      <c r="AR42" s="488" t="n"/>
+      <c r="AS42" s="488" t="n"/>
+      <c r="AT42" s="488" t="n"/>
+      <c r="AU42" s="488" t="n"/>
+      <c r="AV42" s="488" t="n"/>
+      <c r="AW42" s="488" t="n"/>
+      <c r="AX42" s="488" t="n"/>
+      <c r="AY42" s="488" t="n"/>
+      <c r="AZ42" s="488" t="n"/>
+      <c r="BA42" s="488" t="n"/>
+      <c r="BB42" s="488" t="n"/>
+      <c r="BC42" s="488" t="n"/>
+      <c r="BD42" s="493" t="n"/>
+    </row>
+    <row r="43" ht="4" customHeight="1" s="264">
+      <c r="A43" s="469" t="n"/>
+      <c r="B43" s="26" t="n"/>
+      <c r="C43" s="26" t="n"/>
+      <c r="D43" s="26" t="n"/>
+      <c r="E43" s="26" t="n"/>
+      <c r="F43" s="26" t="n"/>
+      <c r="G43" s="26" t="n"/>
+      <c r="H43" s="26" t="n"/>
+      <c r="I43" s="26" t="n"/>
+      <c r="J43" s="26" t="n"/>
+      <c r="K43" s="26" t="n"/>
+      <c r="L43" s="26" t="n"/>
+      <c r="M43" s="26" t="n"/>
+      <c r="N43" s="26" t="n"/>
+      <c r="O43" s="26" t="n"/>
+      <c r="P43" s="26" t="n"/>
+      <c r="Q43" s="26" t="n"/>
+      <c r="R43" s="26" t="n"/>
+      <c r="S43" s="26" t="n"/>
+      <c r="T43" s="26" t="n"/>
+      <c r="U43" s="26" t="n"/>
+      <c r="V43" s="26" t="n"/>
+      <c r="W43" s="26" t="n"/>
+      <c r="X43" s="26" t="n"/>
+      <c r="Y43" s="26" t="n"/>
+      <c r="Z43" s="26" t="n"/>
+      <c r="AA43" s="26" t="n"/>
+      <c r="AB43" s="26" t="n"/>
+      <c r="AC43" s="26" t="n"/>
+      <c r="AD43" s="26" t="n"/>
+      <c r="AE43" s="26" t="n"/>
+      <c r="AF43" s="26" t="n"/>
+      <c r="AG43" s="26" t="n"/>
+      <c r="AH43" s="26" t="n"/>
+      <c r="AI43" s="26" t="n"/>
+      <c r="AJ43" s="26" t="n"/>
+      <c r="AK43" s="26" t="n"/>
+      <c r="AL43" s="26" t="n"/>
+      <c r="AM43" s="26" t="n"/>
+      <c r="AN43" s="26" t="n"/>
+      <c r="AO43" s="26" t="n"/>
+      <c r="AP43" s="26" t="n"/>
+      <c r="AQ43" s="26" t="n"/>
+      <c r="AR43" s="26" t="n"/>
+      <c r="AS43" s="26" t="n"/>
+      <c r="AT43" s="26" t="n"/>
+      <c r="AU43" s="26" t="n"/>
+      <c r="AV43" s="26" t="n"/>
+      <c r="AW43" s="26" t="n"/>
+      <c r="AX43" s="26" t="n"/>
+      <c r="AY43" s="26" t="n"/>
+      <c r="AZ43" s="26" t="n"/>
+      <c r="BA43" s="26" t="n"/>
+      <c r="BB43" s="26" t="n"/>
+      <c r="BC43" s="26" t="n"/>
+      <c r="BD43" s="26" t="n"/>
+    </row>
+    <row r="44" ht="24" customHeight="1" s="264">
+      <c r="A44" s="512" t="inlineStr">
+        <is>
+          <t>NOTICE — Every dimension, note and GD&amp;T callout on the drawing must carry a unique balloon and one row here. This sheet is the master index for FAI (FRM-311) and in-process inspection (FRM-622). Ref: SOP-301. Retain: life of part. Enter data only in white input cells. Do not add, delete or resize columns/rows.</t>
+        </is>
+      </c>
+      <c r="B44" s="471" t="n"/>
+      <c r="C44" s="471" t="n"/>
+      <c r="D44" s="471" t="n"/>
+      <c r="E44" s="471" t="n"/>
+      <c r="F44" s="471" t="n"/>
+      <c r="G44" s="471" t="n"/>
+      <c r="H44" s="471" t="n"/>
+      <c r="I44" s="471" t="n"/>
+      <c r="J44" s="471" t="n"/>
+      <c r="K44" s="471" t="n"/>
+      <c r="L44" s="471" t="n"/>
+      <c r="M44" s="471" t="n"/>
+      <c r="N44" s="471" t="n"/>
+      <c r="O44" s="471" t="n"/>
+      <c r="P44" s="471" t="n"/>
+      <c r="Q44" s="471" t="n"/>
+      <c r="R44" s="471" t="n"/>
+      <c r="S44" s="471" t="n"/>
+      <c r="T44" s="471" t="n"/>
+      <c r="U44" s="471" t="n"/>
+      <c r="V44" s="471" t="n"/>
+      <c r="W44" s="471" t="n"/>
+      <c r="X44" s="471" t="n"/>
+      <c r="Y44" s="471" t="n"/>
+      <c r="Z44" s="471" t="n"/>
+      <c r="AA44" s="471" t="n"/>
+      <c r="AB44" s="471" t="n"/>
+      <c r="AC44" s="471" t="n"/>
+      <c r="AD44" s="471" t="n"/>
+      <c r="AE44" s="471" t="n"/>
+      <c r="AF44" s="471" t="n"/>
+      <c r="AG44" s="471" t="n"/>
+      <c r="AH44" s="471" t="n"/>
+      <c r="AI44" s="471" t="n"/>
+      <c r="AJ44" s="471" t="n"/>
+      <c r="AK44" s="471" t="n"/>
+      <c r="AL44" s="471" t="n"/>
+      <c r="AM44" s="471" t="n"/>
+      <c r="AN44" s="471" t="n"/>
+      <c r="AO44" s="471" t="n"/>
+      <c r="AP44" s="471" t="n"/>
+      <c r="AQ44" s="471" t="n"/>
+      <c r="AR44" s="471" t="n"/>
+      <c r="AS44" s="471" t="n"/>
+      <c r="AT44" s="471" t="n"/>
+      <c r="AU44" s="471" t="n"/>
+      <c r="AV44" s="471" t="n"/>
+      <c r="AW44" s="471" t="n"/>
+      <c r="AX44" s="471" t="n"/>
+      <c r="AY44" s="471" t="n"/>
+      <c r="AZ44" s="471" t="n"/>
+      <c r="BA44" s="471" t="n"/>
+      <c r="BB44" s="471" t="n"/>
+      <c r="BC44" s="471" t="n"/>
+      <c r="BD44" s="472" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="154">
-    <mergeCell ref="W13:AG13"/>
-    <mergeCell ref="E12:I12"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="AM24:AU24"/>
+  <mergeCells count="194">
+    <mergeCell ref="K35:AB35"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="AE20:AI20"/>
+    <mergeCell ref="U24:AD24"/>
+    <mergeCell ref="U18:AD18"/>
+    <mergeCell ref="H27:T27"/>
     <mergeCell ref="AW2:BD2"/>
-    <mergeCell ref="BA20:BD20"/>
-    <mergeCell ref="W15:AG15"/>
-    <mergeCell ref="AH24:AL24"/>
-    <mergeCell ref="W24:AG24"/>
-    <mergeCell ref="AH18:AL18"/>
-    <mergeCell ref="E14:I14"/>
-    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A43:BD43"/>
+    <mergeCell ref="AJ28:AR28"/>
+    <mergeCell ref="S40:AK42"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="AL39:BD39"/>
+    <mergeCell ref="AE22:AI22"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="AE31:AI31"/>
+    <mergeCell ref="AJ30:AR30"/>
+    <mergeCell ref="AY20:BD20"/>
     <mergeCell ref="AQ5:AV5"/>
-    <mergeCell ref="J17:V17"/>
+    <mergeCell ref="AE21:AI21"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="AY29:BD29"/>
     <mergeCell ref="AW3:BD3"/>
-    <mergeCell ref="BA12:BD12"/>
-    <mergeCell ref="E13:I13"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="BA21:BD21"/>
-    <mergeCell ref="AH10:AL10"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A34:J34"/>
+    <mergeCell ref="AS28:AX28"/>
     <mergeCell ref="AQ4:AV4"/>
-    <mergeCell ref="J19:V19"/>
+    <mergeCell ref="AE23:AI23"/>
+    <mergeCell ref="AY31:BD31"/>
+    <mergeCell ref="D22:G22"/>
     <mergeCell ref="AW5:BD5"/>
-    <mergeCell ref="E15:I15"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="A36:J36"/>
     <mergeCell ref="L2:AP4"/>
-    <mergeCell ref="BA23:BD23"/>
+    <mergeCell ref="U27:AD27"/>
     <mergeCell ref="AQ6:AV6"/>
-    <mergeCell ref="J9:V9"/>
-    <mergeCell ref="AV19:AZ19"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="AV9:AZ9"/>
-    <mergeCell ref="E16:I16"/>
-    <mergeCell ref="BA18:BD18"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="AM14:AU14"/>
-    <mergeCell ref="AV20:AZ20"/>
-    <mergeCell ref="W14:AG14"/>
-    <mergeCell ref="AH22:AL22"/>
-    <mergeCell ref="E18:I18"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="AH12:AL12"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="AH21:AL21"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="BA25:BD25"/>
-    <mergeCell ref="AH14:AL14"/>
+    <mergeCell ref="AY15:BD15"/>
+    <mergeCell ref="U30:AD30"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="U17:AD17"/>
+    <mergeCell ref="AY21:BD21"/>
+    <mergeCell ref="AY26:BD26"/>
+    <mergeCell ref="AY23:BD23"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="AJ27:AR27"/>
+    <mergeCell ref="AE27:AI27"/>
+    <mergeCell ref="U21:AD21"/>
+    <mergeCell ref="AJ17:AR17"/>
+    <mergeCell ref="AS25:AX25"/>
+    <mergeCell ref="AE25:AI25"/>
+    <mergeCell ref="A38:BD38"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="AJ19:AR19"/>
+    <mergeCell ref="AS27:AX27"/>
+    <mergeCell ref="A13:BD13"/>
+    <mergeCell ref="A44:BD44"/>
     <mergeCell ref="AQ2:AV2"/>
-    <mergeCell ref="AH23:AL23"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="BA9:BD9"/>
-    <mergeCell ref="J18:V18"/>
-    <mergeCell ref="E20:I20"/>
-    <mergeCell ref="AM10:AU10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="BA11:BD11"/>
-    <mergeCell ref="AM16:AU16"/>
-    <mergeCell ref="AM25:AU25"/>
-    <mergeCell ref="J10:V10"/>
-    <mergeCell ref="W16:AG16"/>
+    <mergeCell ref="H15:T15"/>
+    <mergeCell ref="AS17:AX17"/>
+    <mergeCell ref="H24:T24"/>
+    <mergeCell ref="H18:T18"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="U26:AD26"/>
+    <mergeCell ref="AY19:BD19"/>
+    <mergeCell ref="AM10:BD10"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="AS19:AX19"/>
+    <mergeCell ref="H26:T26"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="AJ20:AR20"/>
+    <mergeCell ref="AY25:BD25"/>
+    <mergeCell ref="AJ29:AR29"/>
+    <mergeCell ref="AY30:BD30"/>
     <mergeCell ref="A7:BD7"/>
-    <mergeCell ref="AV10:AZ10"/>
-    <mergeCell ref="AM18:AU18"/>
-    <mergeCell ref="AV24:AZ24"/>
-    <mergeCell ref="A27:BD27"/>
-    <mergeCell ref="W18:AG18"/>
-    <mergeCell ref="AM17:AU17"/>
-    <mergeCell ref="BA13:BD13"/>
-    <mergeCell ref="AH16:AL16"/>
-    <mergeCell ref="W17:AG17"/>
-    <mergeCell ref="W11:AG11"/>
-    <mergeCell ref="AH25:AL25"/>
-    <mergeCell ref="AM22:AU22"/>
-    <mergeCell ref="AM19:AU19"/>
+    <mergeCell ref="AE29:AI29"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="H25:T25"/>
+    <mergeCell ref="AJ22:AR22"/>
+    <mergeCell ref="AJ31:AR31"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="AS30:AX30"/>
+    <mergeCell ref="AM36:BD36"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="U16:AD16"/>
+    <mergeCell ref="U25:AD25"/>
+    <mergeCell ref="AS20:AX20"/>
+    <mergeCell ref="A39:R39"/>
+    <mergeCell ref="AJ21:AR21"/>
+    <mergeCell ref="AS29:AX29"/>
+    <mergeCell ref="AE15:AI15"/>
+    <mergeCell ref="K9:AB9"/>
+    <mergeCell ref="H17:T17"/>
+    <mergeCell ref="AE24:AI24"/>
+    <mergeCell ref="A33:BD33"/>
+    <mergeCell ref="AC35:AL35"/>
     <mergeCell ref="L5:AP5"/>
-    <mergeCell ref="J20:V20"/>
-    <mergeCell ref="BA15:BD15"/>
-    <mergeCell ref="BA24:BD24"/>
-    <mergeCell ref="W19:AG19"/>
-    <mergeCell ref="J22:V22"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="W25:AG25"/>
-    <mergeCell ref="J12:V12"/>
-    <mergeCell ref="AV22:AZ22"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="J21:V21"/>
-    <mergeCell ref="BA16:BD16"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="AM20:AU20"/>
-    <mergeCell ref="AV12:AZ12"/>
+    <mergeCell ref="AS22:AX22"/>
+    <mergeCell ref="AJ23:AR23"/>
+    <mergeCell ref="AS31:AX31"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="U28:AD28"/>
+    <mergeCell ref="AC34:AL34"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="K11:AB11"/>
+    <mergeCell ref="H19:T19"/>
+    <mergeCell ref="AE26:AI26"/>
+    <mergeCell ref="AM34:BD34"/>
+    <mergeCell ref="AS21:AX21"/>
+    <mergeCell ref="H28:T28"/>
+    <mergeCell ref="AC9:AL9"/>
+    <mergeCell ref="AE16:AI16"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="AY24:BD24"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="U20:AD20"/>
+    <mergeCell ref="AJ18:AR18"/>
+    <mergeCell ref="AC11:AL11"/>
+    <mergeCell ref="U29:AD29"/>
+    <mergeCell ref="U23:AD23"/>
+    <mergeCell ref="AE18:AI18"/>
+    <mergeCell ref="A14:BD14"/>
     <mergeCell ref="AW4:BD4"/>
-    <mergeCell ref="AH20:AL20"/>
-    <mergeCell ref="AV21:AZ21"/>
-    <mergeCell ref="E10:I10"/>
-    <mergeCell ref="J23:V23"/>
-    <mergeCell ref="E19:I19"/>
-    <mergeCell ref="AV14:AZ14"/>
-    <mergeCell ref="AV23:AZ23"/>
-    <mergeCell ref="E9:I9"/>
-    <mergeCell ref="AM12:AU12"/>
-    <mergeCell ref="AV13:AZ13"/>
-    <mergeCell ref="AM21:AU21"/>
-    <mergeCell ref="AH15:AL15"/>
-    <mergeCell ref="BA22:BD22"/>
-    <mergeCell ref="W21:AG21"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="A26:BD26"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="J16:V16"/>
-    <mergeCell ref="J11:V11"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="AS16:AX16"/>
+    <mergeCell ref="H23:T23"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="U22:AD22"/>
+    <mergeCell ref="U31:AD31"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="AE17:AI17"/>
+    <mergeCell ref="U15:AD15"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="AY16:BD16"/>
+    <mergeCell ref="AJ25:AR25"/>
+    <mergeCell ref="AE19:AI19"/>
+    <mergeCell ref="K10:AB10"/>
+    <mergeCell ref="AE28:AI28"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="AY18:BD18"/>
+    <mergeCell ref="K34:AB34"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="AE30:AI30"/>
+    <mergeCell ref="AY22:BD22"/>
+    <mergeCell ref="K36:AB36"/>
+    <mergeCell ref="D28:G28"/>
     <mergeCell ref="A8:BD8"/>
-    <mergeCell ref="J25:V25"/>
-    <mergeCell ref="BA14:BD14"/>
-    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="AC10:AL10"/>
     <mergeCell ref="AQ3:AV3"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="AV16:AZ16"/>
-    <mergeCell ref="W10:AG10"/>
-    <mergeCell ref="AV25:AZ25"/>
-    <mergeCell ref="AM9:AU9"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="AV18:AZ18"/>
-    <mergeCell ref="AH17:AL17"/>
-    <mergeCell ref="AM11:AU11"/>
+    <mergeCell ref="H22:T22"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A35:J35"/>
+    <mergeCell ref="AM9:BD9"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="AY28:BD28"/>
+    <mergeCell ref="U19:AD19"/>
+    <mergeCell ref="K12:AB12"/>
+    <mergeCell ref="AC36:AL36"/>
+    <mergeCell ref="AJ15:AR15"/>
     <mergeCell ref="L6:AP6"/>
-    <mergeCell ref="AV17:AZ17"/>
-    <mergeCell ref="AV11:AZ11"/>
-    <mergeCell ref="AH19:AL19"/>
-    <mergeCell ref="W20:AG20"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="AJ24:AR24"/>
+    <mergeCell ref="AM11:BD11"/>
+    <mergeCell ref="AS23:AX23"/>
+    <mergeCell ref="H30:T30"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="H20:T20"/>
     <mergeCell ref="AW6:BD6"/>
-    <mergeCell ref="J14:V14"/>
-    <mergeCell ref="AH9:AL9"/>
-    <mergeCell ref="AM15:AU15"/>
-    <mergeCell ref="W22:AG22"/>
-    <mergeCell ref="J13:V13"/>
-    <mergeCell ref="BA17:BD17"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="AH11:AL11"/>
-    <mergeCell ref="W12:AG12"/>
-    <mergeCell ref="J15:V15"/>
-    <mergeCell ref="BA10:BD10"/>
-    <mergeCell ref="J24:V24"/>
-    <mergeCell ref="W9:AG9"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="BA19:BD19"/>
+    <mergeCell ref="H29:T29"/>
+    <mergeCell ref="AM35:BD35"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="AJ26:AR26"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="AS15:AX15"/>
+    <mergeCell ref="AJ16:AR16"/>
+    <mergeCell ref="AL40:BD42"/>
+    <mergeCell ref="AM12:BD12"/>
+    <mergeCell ref="AS24:AX24"/>
+    <mergeCell ref="H31:T31"/>
+    <mergeCell ref="AC12:AL12"/>
+    <mergeCell ref="AS18:AX18"/>
+    <mergeCell ref="S39:AK39"/>
+    <mergeCell ref="AY27:BD27"/>
+    <mergeCell ref="H21:T21"/>
+    <mergeCell ref="A37:BD37"/>
+    <mergeCell ref="AS26:AX26"/>
     <mergeCell ref="A2:K6"/>
-    <mergeCell ref="AV15:AZ15"/>
-    <mergeCell ref="AM23:AU23"/>
-    <mergeCell ref="AM13:AU13"/>
-    <mergeCell ref="W23:AG23"/>
-    <mergeCell ref="E22:I22"/>
-    <mergeCell ref="AH13:AL13"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="A40:R42"/>
+    <mergeCell ref="A32:BD32"/>
+    <mergeCell ref="AY17:BD17"/>
+    <mergeCell ref="H16:T16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>